<commit_message>
Alphabetic insertion of new students
</commit_message>
<xml_diff>
--- a/Testing/basic_sequence/workbook.xlsx
+++ b/Testing/basic_sequence/workbook.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Pavan Rauch\git\Truancy-Local\Testing\basic_sequence\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44992D27-A81E-457B-A09F-F7AC42C83882}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BF430B2-4C74-47B1-893B-EB530D8C29F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Urbana Elementary (Before)" sheetId="4" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="49">
   <si>
     <t>Last Name</t>
   </si>
@@ -80,100 +80,100 @@
     <t>3rd</t>
   </si>
   <si>
+    <t>John</t>
+  </si>
+  <si>
+    <t>Smith</t>
+  </si>
+  <si>
+    <t>Jane</t>
+  </si>
+  <si>
+    <t>Johnson</t>
+  </si>
+  <si>
+    <t>Michael</t>
+  </si>
+  <si>
+    <t>Davis</t>
+  </si>
+  <si>
+    <t>Emily</t>
+  </si>
+  <si>
+    <t>Brown</t>
+  </si>
+  <si>
+    <t>David</t>
+  </si>
+  <si>
+    <t>Martinez</t>
+  </si>
+  <si>
+    <t>Olivia</t>
+  </si>
+  <si>
+    <t>Lee</t>
+  </si>
+  <si>
+    <t>Christopher</t>
+  </si>
+  <si>
+    <t>Rodriguez</t>
+  </si>
+  <si>
+    <t>Sophia</t>
+  </si>
+  <si>
+    <t>extra comment</t>
+  </si>
+  <si>
+    <t>this is a comment</t>
+  </si>
+  <si>
+    <t>another comment</t>
+  </si>
+  <si>
+    <t>commenting</t>
+  </si>
+  <si>
+    <t>important comment</t>
+  </si>
+  <si>
+    <t>withdrawal</t>
+  </si>
+  <si>
+    <t>1/7/2025 Unexcused Absences</t>
+  </si>
+  <si>
+    <t>1/28/2025 Unexcused Absences</t>
+  </si>
+  <si>
+    <t>Wilson</t>
+  </si>
+  <si>
+    <t>Sarah</t>
+  </si>
+  <si>
+    <t>Taylor</t>
+  </si>
+  <si>
+    <t>James</t>
+  </si>
+  <si>
+    <t>1/7/2025 Excused Absences</t>
+  </si>
+  <si>
+    <t>1/14/2025 Excused Absences</t>
+  </si>
+  <si>
+    <t>1/23/2025 Excused Absences</t>
+  </si>
+  <si>
+    <t>1/28/2025 Excused Absences</t>
+  </si>
+  <si>
     <t>Doe</t>
-  </si>
-  <si>
-    <t>John</t>
-  </si>
-  <si>
-    <t>Smith</t>
-  </si>
-  <si>
-    <t>Jane</t>
-  </si>
-  <si>
-    <t>Johnson</t>
-  </si>
-  <si>
-    <t>Michael</t>
-  </si>
-  <si>
-    <t>Davis</t>
-  </si>
-  <si>
-    <t>Emily</t>
-  </si>
-  <si>
-    <t>Brown</t>
-  </si>
-  <si>
-    <t>David</t>
-  </si>
-  <si>
-    <t>Martinez</t>
-  </si>
-  <si>
-    <t>Olivia</t>
-  </si>
-  <si>
-    <t>Lee</t>
-  </si>
-  <si>
-    <t>Christopher</t>
-  </si>
-  <si>
-    <t>Rodriguez</t>
-  </si>
-  <si>
-    <t>Sophia</t>
-  </si>
-  <si>
-    <t>extra comment</t>
-  </si>
-  <si>
-    <t>this is a comment</t>
-  </si>
-  <si>
-    <t>another comment</t>
-  </si>
-  <si>
-    <t>commenting</t>
-  </si>
-  <si>
-    <t>important comment</t>
-  </si>
-  <si>
-    <t>withdrawal</t>
-  </si>
-  <si>
-    <t>1/7/2025 Unexcused Absences</t>
-  </si>
-  <si>
-    <t>1/28/2025 Unexcused Absences</t>
-  </si>
-  <si>
-    <t>Wilson</t>
-  </si>
-  <si>
-    <t>Sarah</t>
-  </si>
-  <si>
-    <t>Taylor</t>
-  </si>
-  <si>
-    <t>James</t>
-  </si>
-  <si>
-    <t>1/7/2025 Excused Absences</t>
-  </si>
-  <si>
-    <t>1/14/2025 Excused Absences</t>
-  </si>
-  <si>
-    <t>1/23/2025 Excused Absences</t>
-  </si>
-  <si>
-    <t>1/28/2025 Excused Absences</t>
   </si>
 </sst>
 </file>
@@ -218,7 +218,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -246,6 +246,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -347,10 +353,12 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -625,9 +633,7 @@
     <col min="5" max="5" width="6.140625" style="1" customWidth="1"/>
     <col min="6" max="6" width="11.42578125" style="2" customWidth="1"/>
     <col min="7" max="7" width="10.28515625" style="2" customWidth="1"/>
-    <col min="8" max="8" width="12" customWidth="1"/>
-    <col min="9" max="9" width="12" style="28" customWidth="1"/>
-    <col min="10" max="14" width="12" customWidth="1"/>
+    <col min="8" max="14" width="12" customWidth="1"/>
     <col min="15" max="15" width="32.28515625" style="2" customWidth="1"/>
   </cols>
   <sheetData>
@@ -657,19 +663,19 @@
         <v>7</v>
       </c>
       <c r="I1" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="J1" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="K1" s="7" t="s">
         <v>45</v>
-      </c>
-      <c r="J1" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="K1" s="7" t="s">
-        <v>46</v>
       </c>
       <c r="L1" s="7" t="s">
         <v>8</v>
       </c>
       <c r="M1" s="7" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="N1" s="7" t="s">
         <v>9</v>
@@ -680,16 +686,16 @@
     </row>
     <row r="2" spans="1:16" ht="15" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="C2" s="9">
-        <v>117031</v>
+        <v>118678</v>
       </c>
       <c r="D2" s="11">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E2" s="10" t="s">
         <v>16</v>
@@ -699,121 +705,117 @@
       <c r="H2" s="24">
         <v>0</v>
       </c>
-      <c r="I2" s="26">
-        <v>0</v>
-      </c>
-      <c r="J2" s="26">
-        <v>40</v>
-      </c>
-      <c r="K2" s="26">
-        <v>6</v>
-      </c>
-      <c r="L2" s="26">
-        <v>40</v>
-      </c>
-      <c r="M2" s="26">
-        <v>6</v>
-      </c>
-      <c r="N2" s="26">
-        <v>52</v>
-      </c>
-      <c r="O2" s="13" t="s">
-        <v>34</v>
-      </c>
+      <c r="I2" s="22">
+        <v>0</v>
+      </c>
+      <c r="J2" s="22">
+        <v>0</v>
+      </c>
+      <c r="K2" s="22">
+        <v>0</v>
+      </c>
+      <c r="L2" s="22">
+        <v>10</v>
+      </c>
+      <c r="M2" s="22">
+        <v>0</v>
+      </c>
+      <c r="N2" s="22">
+        <v>10</v>
+      </c>
+      <c r="O2" s="13"/>
     </row>
     <row r="3" spans="1:16" ht="15" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C3" s="9">
-        <v>116157</v>
+        <v>118245</v>
       </c>
       <c r="D3" s="11">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="F3" s="12"/>
       <c r="G3" s="12"/>
       <c r="H3" s="24">
         <v>0</v>
       </c>
-      <c r="I3" s="27">
-        <v>0</v>
-      </c>
-      <c r="J3" s="27">
-        <v>23.15</v>
-      </c>
-      <c r="K3" s="27">
-        <v>5</v>
-      </c>
-      <c r="L3" s="27">
-        <v>23.15</v>
-      </c>
-      <c r="M3" s="26">
-        <v>5</v>
-      </c>
-      <c r="N3" s="26">
-        <v>43.15</v>
+      <c r="I3" s="22">
+        <v>0</v>
+      </c>
+      <c r="J3" s="22"/>
+      <c r="K3" s="22">
+        <v>15</v>
+      </c>
+      <c r="L3" s="22">
+        <v>0</v>
+      </c>
+      <c r="M3" s="22">
+        <v>15</v>
+      </c>
+      <c r="N3" s="22">
+        <v>0</v>
       </c>
       <c r="O3" s="13"/>
     </row>
     <row r="4" spans="1:16" ht="15" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="C4" s="9">
-        <v>115936</v>
+        <v>117031</v>
       </c>
       <c r="D4" s="11">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="F4" s="12"/>
       <c r="G4" s="12"/>
       <c r="H4" s="24">
         <v>0</v>
       </c>
-      <c r="I4" s="27">
-        <v>20</v>
-      </c>
-      <c r="J4" s="27">
-        <v>0</v>
-      </c>
-      <c r="K4" s="27">
-        <v>20</v>
-      </c>
-      <c r="L4" s="27">
-        <v>15</v>
-      </c>
-      <c r="M4" s="27">
-        <v>20</v>
-      </c>
-      <c r="N4" s="27">
-        <v>15</v>
+      <c r="I4" s="26">
+        <v>0</v>
+      </c>
+      <c r="J4" s="26">
+        <v>40</v>
+      </c>
+      <c r="K4" s="26">
+        <v>6</v>
+      </c>
+      <c r="L4" s="26">
+        <v>40</v>
+      </c>
+      <c r="M4" s="26">
+        <v>6</v>
+      </c>
+      <c r="N4" s="26">
+        <v>52</v>
       </c>
       <c r="O4" s="13" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="5" spans="1:16" ht="15" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="C5" s="9">
-        <v>118245</v>
+        <v>122965</v>
       </c>
       <c r="D5" s="11">
         <v>7</v>
@@ -826,195 +828,199 @@
       <c r="H5" s="24">
         <v>0</v>
       </c>
-      <c r="I5" s="27">
-        <v>0</v>
-      </c>
-      <c r="J5" s="27"/>
-      <c r="K5" s="27">
+      <c r="I5" s="22">
+        <v>10</v>
+      </c>
+      <c r="J5" s="22">
         <v>15</v>
       </c>
-      <c r="L5" s="27">
-        <v>0</v>
-      </c>
-      <c r="M5" s="27">
+      <c r="K5" s="22">
+        <v>10</v>
+      </c>
+      <c r="L5" s="22">
         <v>15</v>
       </c>
-      <c r="N5" s="27">
-        <v>0</v>
-      </c>
-      <c r="O5" s="13"/>
+      <c r="M5" s="26">
+        <v>10</v>
+      </c>
+      <c r="N5" s="26">
+        <v>34</v>
+      </c>
+      <c r="O5" s="15" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="6" spans="1:16" ht="15" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C6" s="9">
-        <v>118678</v>
+        <v>121874</v>
       </c>
       <c r="D6" s="11">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="F6" s="12"/>
       <c r="G6" s="12"/>
       <c r="H6" s="24">
-        <v>0</v>
-      </c>
-      <c r="I6" s="27">
-        <v>0</v>
-      </c>
-      <c r="J6" s="27">
-        <v>0</v>
-      </c>
-      <c r="K6" s="27">
-        <v>0</v>
-      </c>
-      <c r="L6" s="27">
-        <v>10</v>
-      </c>
-      <c r="M6" s="27">
-        <v>0</v>
-      </c>
-      <c r="N6" s="27">
-        <v>10</v>
-      </c>
-      <c r="O6" s="13"/>
+        <v>8.25</v>
+      </c>
+      <c r="I6" s="26">
+        <v>42.33</v>
+      </c>
+      <c r="J6" s="26">
+        <v>14</v>
+      </c>
+      <c r="K6" s="26">
+        <v>42.33</v>
+      </c>
+      <c r="L6" s="26">
+        <v>14</v>
+      </c>
+      <c r="M6" s="26">
+        <v>42.33</v>
+      </c>
+      <c r="N6" s="26">
+        <v>32</v>
+      </c>
+      <c r="O6" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="P6" s="14" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="7" spans="1:16" ht="15" x14ac:dyDescent="0.25">
-      <c r="A7" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="B7" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="C7" s="9">
-        <v>121874</v>
-      </c>
-      <c r="D7" s="11">
-        <v>8</v>
-      </c>
-      <c r="E7" s="10" t="s">
+      <c r="A7" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="B7" s="18" t="s">
+        <v>31</v>
+      </c>
+      <c r="C7" s="17">
+        <v>125674</v>
+      </c>
+      <c r="D7" s="19">
+        <v>9</v>
+      </c>
+      <c r="E7" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="F7" s="12"/>
-      <c r="G7" s="12"/>
-      <c r="H7" s="24">
-        <v>8.25</v>
-      </c>
-      <c r="I7" s="26">
-        <v>42.33</v>
-      </c>
-      <c r="J7" s="26">
+      <c r="F7" s="20"/>
+      <c r="G7" s="20"/>
+      <c r="H7" s="25">
+        <v>0</v>
+      </c>
+      <c r="I7" s="23">
+        <v>13</v>
+      </c>
+      <c r="J7" s="23">
+        <v>55</v>
+      </c>
+      <c r="K7" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="K7" s="26">
-        <v>42.33</v>
-      </c>
-      <c r="L7" s="26">
+      <c r="L7" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="M7" s="26">
-        <v>42.33</v>
-      </c>
-      <c r="N7" s="26">
-        <v>32</v>
-      </c>
-      <c r="O7" s="13" t="s">
-        <v>36</v>
-      </c>
-      <c r="P7" s="14" t="s">
-        <v>33</v>
+      <c r="M7" s="23" t="s">
+        <v>14</v>
+      </c>
+      <c r="N7" s="23" t="s">
+        <v>14</v>
+      </c>
+      <c r="O7" s="21" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="8" spans="1:16" ht="15" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>30</v>
+        <v>19</v>
       </c>
       <c r="C8" s="9">
-        <v>122965</v>
+        <v>116157</v>
       </c>
       <c r="D8" s="11">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="F8" s="12"/>
       <c r="G8" s="12"/>
       <c r="H8" s="24">
         <v>0</v>
       </c>
-      <c r="I8" s="27">
-        <v>10</v>
-      </c>
-      <c r="J8" s="27">
+      <c r="I8" s="22">
+        <v>0</v>
+      </c>
+      <c r="J8" s="22">
+        <v>23.15</v>
+      </c>
+      <c r="K8" s="22">
+        <v>5</v>
+      </c>
+      <c r="L8" s="22">
+        <v>23.15</v>
+      </c>
+      <c r="M8" s="26">
+        <v>5</v>
+      </c>
+      <c r="N8" s="26">
+        <v>43.15</v>
+      </c>
+      <c r="O8" s="13"/>
+    </row>
+    <row r="9" spans="1:16" ht="15" x14ac:dyDescent="0.25">
+      <c r="A9" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="B9" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="C9" s="9">
+        <v>115936</v>
+      </c>
+      <c r="D9" s="11">
+        <v>8</v>
+      </c>
+      <c r="E9" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="F9" s="12"/>
+      <c r="G9" s="12"/>
+      <c r="H9" s="24">
+        <v>0</v>
+      </c>
+      <c r="I9" s="22">
+        <v>20</v>
+      </c>
+      <c r="J9" s="22">
+        <v>0</v>
+      </c>
+      <c r="K9" s="22">
+        <v>20</v>
+      </c>
+      <c r="L9" s="22">
         <v>15</v>
       </c>
-      <c r="K8" s="27">
-        <v>10</v>
-      </c>
-      <c r="L8" s="27">
+      <c r="M9" s="22">
+        <v>20</v>
+      </c>
+      <c r="N9" s="22">
         <v>15</v>
       </c>
-      <c r="M8" s="26">
-        <v>10</v>
-      </c>
-      <c r="N8" s="26">
+      <c r="O9" s="13" t="s">
         <v>34</v>
-      </c>
-      <c r="O8" s="15" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="9" spans="1:16" ht="15" x14ac:dyDescent="0.25">
-      <c r="A9" s="17" t="s">
-        <v>31</v>
-      </c>
-      <c r="B9" s="18" t="s">
-        <v>32</v>
-      </c>
-      <c r="C9" s="17">
-        <v>125674</v>
-      </c>
-      <c r="D9" s="19">
-        <v>9</v>
-      </c>
-      <c r="E9" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="F9" s="20"/>
-      <c r="G9" s="20"/>
-      <c r="H9" s="25">
-        <v>0</v>
-      </c>
-      <c r="I9" s="23">
-        <v>13</v>
-      </c>
-      <c r="J9" s="23">
-        <v>55</v>
-      </c>
-      <c r="K9" s="23" t="s">
-        <v>14</v>
-      </c>
-      <c r="L9" s="23" t="s">
-        <v>14</v>
-      </c>
-      <c r="M9" s="23" t="s">
-        <v>14</v>
-      </c>
-      <c r="N9" s="23" t="s">
-        <v>14</v>
-      </c>
-      <c r="O9" s="21" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="10" spans="1:16" ht="15" x14ac:dyDescent="0.25">
@@ -1026,7 +1032,7 @@
       <c r="F10" s="12"/>
       <c r="G10" s="12"/>
       <c r="H10" s="24"/>
-      <c r="I10" s="27"/>
+      <c r="I10" s="22"/>
       <c r="J10" s="22"/>
       <c r="K10" s="22"/>
       <c r="L10" s="22"/>
@@ -1043,7 +1049,7 @@
       <c r="F11" s="12"/>
       <c r="G11" s="12"/>
       <c r="H11" s="24"/>
-      <c r="I11" s="27"/>
+      <c r="I11" s="22"/>
       <c r="J11" s="22"/>
       <c r="K11" s="22"/>
       <c r="L11" s="22"/>
@@ -1154,6 +1160,9 @@
       <c r="H45" s="16"/>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:P9">
+    <sortCondition ref="A2:A9"/>
+  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup fitToHeight="0" orientation="landscape" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
@@ -1174,9 +1183,7 @@
     <col min="5" max="5" width="6.140625" style="1" customWidth="1"/>
     <col min="6" max="6" width="11.42578125" style="2" customWidth="1"/>
     <col min="7" max="7" width="10.28515625" style="2" customWidth="1"/>
-    <col min="8" max="8" width="12" customWidth="1"/>
-    <col min="9" max="9" width="12" style="28" customWidth="1"/>
-    <col min="10" max="16" width="12" customWidth="1"/>
+    <col min="8" max="16" width="12" customWidth="1"/>
     <col min="17" max="17" width="32.28515625" style="2" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1206,28 +1213,28 @@
         <v>7</v>
       </c>
       <c r="I1" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="J1" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="K1" s="7" t="s">
         <v>45</v>
-      </c>
-      <c r="J1" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="K1" s="7" t="s">
-        <v>46</v>
       </c>
       <c r="L1" s="7" t="s">
         <v>8</v>
       </c>
       <c r="M1" s="7" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="N1" s="7" t="s">
         <v>9</v>
       </c>
       <c r="O1" s="7" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="P1" s="7" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="Q1" s="8" t="s">
         <v>10</v>
@@ -1235,16 +1242,16 @@
     </row>
     <row r="2" spans="1:18" ht="15" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="C2" s="9">
-        <v>117031</v>
+        <v>118678</v>
       </c>
       <c r="D2" s="11">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E2" s="10" t="s">
         <v>16</v>
@@ -1252,230 +1259,218 @@
       <c r="F2" s="12"/>
       <c r="G2" s="12"/>
       <c r="H2" s="24">
-        <v>19.399999999999999</v>
-      </c>
-      <c r="I2" s="26">
-        <v>0</v>
-      </c>
-      <c r="J2" s="26">
-        <v>40</v>
-      </c>
-      <c r="K2" s="26">
-        <v>6</v>
-      </c>
-      <c r="L2" s="26">
-        <v>40</v>
-      </c>
-      <c r="M2" s="26">
-        <v>6</v>
-      </c>
-      <c r="N2" s="26">
-        <v>52</v>
-      </c>
-      <c r="O2" s="26">
-        <v>6</v>
-      </c>
-      <c r="P2" s="26">
-        <v>62</v>
-      </c>
-      <c r="Q2" s="13" t="s">
-        <v>34</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="I2" s="22">
+        <v>0</v>
+      </c>
+      <c r="J2" s="22">
+        <v>0</v>
+      </c>
+      <c r="K2" s="22">
+        <v>0</v>
+      </c>
+      <c r="L2" s="22">
+        <v>10</v>
+      </c>
+      <c r="M2" s="22">
+        <v>0</v>
+      </c>
+      <c r="N2" s="22">
+        <v>10</v>
+      </c>
+      <c r="O2" s="22">
+        <v>2</v>
+      </c>
+      <c r="P2" s="22">
+        <v>10</v>
+      </c>
+      <c r="Q2" s="13"/>
     </row>
     <row r="3" spans="1:18" ht="15" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C3" s="9">
-        <v>116157</v>
+        <v>118245</v>
       </c>
       <c r="D3" s="11">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="F3" s="12"/>
       <c r="G3" s="12"/>
       <c r="H3" s="24">
         <v>0</v>
       </c>
-      <c r="I3" s="27">
-        <v>0</v>
-      </c>
-      <c r="J3" s="27">
-        <v>23.15</v>
-      </c>
-      <c r="K3" s="27">
-        <v>5</v>
-      </c>
-      <c r="L3" s="27">
-        <v>23.15</v>
-      </c>
-      <c r="M3" s="26">
-        <v>5</v>
-      </c>
-      <c r="N3" s="26">
-        <v>43.15</v>
+      <c r="I3" s="22">
+        <v>0</v>
+      </c>
+      <c r="J3" s="22"/>
+      <c r="K3" s="22">
+        <v>15</v>
+      </c>
+      <c r="L3" s="22">
+        <v>0</v>
+      </c>
+      <c r="M3" s="22">
+        <v>15</v>
+      </c>
+      <c r="N3" s="22">
+        <v>0</v>
       </c>
       <c r="O3" s="26">
-        <v>6</v>
+        <v>50</v>
       </c>
       <c r="P3" s="26">
-        <v>50.15</v>
+        <v>0</v>
       </c>
       <c r="Q3" s="13"/>
     </row>
     <row r="4" spans="1:18" ht="15" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="B4" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="B4" s="10" t="s">
-        <v>18</v>
-      </c>
       <c r="C4" s="9">
-        <v>115936</v>
+        <v>120451</v>
       </c>
       <c r="D4" s="11">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F4" s="12"/>
       <c r="G4" s="12"/>
       <c r="H4" s="24">
         <v>0</v>
       </c>
-      <c r="I4" s="27">
-        <v>20</v>
-      </c>
-      <c r="J4" s="27">
-        <v>0</v>
-      </c>
-      <c r="K4" s="27">
-        <v>20</v>
-      </c>
-      <c r="L4" s="27">
-        <v>15</v>
-      </c>
-      <c r="M4" s="27">
-        <v>20</v>
-      </c>
-      <c r="N4" s="27">
-        <v>15</v>
-      </c>
-      <c r="O4" s="27">
-        <v>35</v>
-      </c>
-      <c r="P4" s="27">
-        <v>0</v>
-      </c>
-      <c r="Q4" s="13" t="s">
-        <v>35</v>
-      </c>
+      <c r="I4" s="22"/>
+      <c r="J4" s="22"/>
+      <c r="K4" s="22"/>
+      <c r="L4" s="22"/>
+      <c r="M4" s="22"/>
+      <c r="N4" s="22"/>
+      <c r="O4" s="26">
+        <v>19</v>
+      </c>
+      <c r="P4" s="26">
+        <v>22.5</v>
+      </c>
+      <c r="Q4" s="13"/>
     </row>
     <row r="5" spans="1:18" ht="15" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="C5" s="9">
-        <v>118245</v>
+        <v>117031</v>
       </c>
       <c r="D5" s="11">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="F5" s="12"/>
       <c r="G5" s="12"/>
       <c r="H5" s="24">
-        <v>0</v>
-      </c>
-      <c r="I5" s="27">
-        <v>0</v>
-      </c>
-      <c r="J5" s="27"/>
-      <c r="K5" s="27">
-        <v>15</v>
-      </c>
-      <c r="L5" s="27">
-        <v>0</v>
-      </c>
-      <c r="M5" s="27">
-        <v>15</v>
-      </c>
-      <c r="N5" s="27">
-        <v>0</v>
+        <v>19.399999999999999</v>
+      </c>
+      <c r="I5" s="26">
+        <v>0</v>
+      </c>
+      <c r="J5" s="26">
+        <v>40</v>
+      </c>
+      <c r="K5" s="26">
+        <v>6</v>
+      </c>
+      <c r="L5" s="26">
+        <v>40</v>
+      </c>
+      <c r="M5" s="26">
+        <v>6</v>
+      </c>
+      <c r="N5" s="26">
+        <v>52</v>
       </c>
       <c r="O5" s="26">
-        <v>50</v>
+        <v>6</v>
       </c>
       <c r="P5" s="26">
-        <v>0</v>
-      </c>
-      <c r="Q5" s="13"/>
+        <v>62</v>
+      </c>
+      <c r="Q5" s="13" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="6" spans="1:18" ht="15" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="C6" s="9">
-        <v>118678</v>
+        <v>122965</v>
       </c>
       <c r="D6" s="11">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="F6" s="12"/>
       <c r="G6" s="12"/>
       <c r="H6" s="24">
         <v>0</v>
       </c>
-      <c r="I6" s="27">
-        <v>0</v>
-      </c>
-      <c r="J6" s="27">
-        <v>0</v>
-      </c>
-      <c r="K6" s="27">
-        <v>0</v>
-      </c>
-      <c r="L6" s="27">
+      <c r="I6" s="22">
         <v>10</v>
       </c>
-      <c r="M6" s="27">
-        <v>0</v>
-      </c>
-      <c r="N6" s="27">
+      <c r="J6" s="22">
+        <v>15</v>
+      </c>
+      <c r="K6" s="22">
         <v>10</v>
       </c>
-      <c r="O6" s="27">
-        <v>2</v>
-      </c>
-      <c r="P6" s="27">
+      <c r="L6" s="22">
+        <v>15</v>
+      </c>
+      <c r="M6" s="26">
         <v>10</v>
       </c>
-      <c r="Q6" s="13"/>
+      <c r="N6" s="26">
+        <v>34</v>
+      </c>
+      <c r="O6" s="22">
+        <v>10</v>
+      </c>
+      <c r="P6" s="22">
+        <v>15</v>
+      </c>
+      <c r="Q6" s="15" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="7" spans="1:18" ht="15" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="B7" s="10" t="s">
         <v>27</v>
-      </c>
-      <c r="B7" s="10" t="s">
-        <v>28</v>
       </c>
       <c r="C7" s="9">
         <v>121874</v>
@@ -1509,184 +1504,196 @@
       <c r="N7" s="26">
         <v>32</v>
       </c>
-      <c r="O7" s="27" t="s">
+      <c r="O7" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="P7" s="27" t="s">
+      <c r="P7" s="22" t="s">
         <v>14</v>
       </c>
       <c r="Q7" s="13" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="R7" s="14" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="8" spans="1:18" ht="15" x14ac:dyDescent="0.25">
-      <c r="A8" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="B8" s="10" t="s">
+      <c r="A8" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="C8" s="9">
-        <v>122965</v>
-      </c>
-      <c r="D8" s="11">
-        <v>7</v>
-      </c>
-      <c r="E8" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="F8" s="12"/>
-      <c r="G8" s="12"/>
-      <c r="H8" s="24">
-        <v>0</v>
-      </c>
-      <c r="I8" s="27">
-        <v>10</v>
-      </c>
-      <c r="J8" s="27">
+      <c r="B8" s="18" t="s">
+        <v>31</v>
+      </c>
+      <c r="C8" s="17">
+        <v>125674</v>
+      </c>
+      <c r="D8" s="19">
+        <v>9</v>
+      </c>
+      <c r="E8" s="18" t="s">
+        <v>13</v>
+      </c>
+      <c r="F8" s="20"/>
+      <c r="G8" s="20"/>
+      <c r="H8" s="25">
+        <v>0</v>
+      </c>
+      <c r="I8" s="23">
+        <v>13</v>
+      </c>
+      <c r="J8" s="23">
+        <v>55</v>
+      </c>
+      <c r="K8" s="23" t="s">
+        <v>14</v>
+      </c>
+      <c r="L8" s="23" t="s">
+        <v>14</v>
+      </c>
+      <c r="M8" s="23" t="s">
+        <v>14</v>
+      </c>
+      <c r="N8" s="23" t="s">
+        <v>14</v>
+      </c>
+      <c r="O8" s="23" t="s">
+        <v>14</v>
+      </c>
+      <c r="P8" s="23" t="s">
+        <v>14</v>
+      </c>
+      <c r="Q8" s="21" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" ht="15" x14ac:dyDescent="0.25">
+      <c r="A9" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B9" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="C9" s="9">
+        <v>116157</v>
+      </c>
+      <c r="D9" s="11">
+        <v>12</v>
+      </c>
+      <c r="E9" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="K8" s="27">
-        <v>10</v>
-      </c>
-      <c r="L8" s="27">
-        <v>15</v>
-      </c>
-      <c r="M8" s="26">
-        <v>10</v>
-      </c>
-      <c r="N8" s="26">
-        <v>34</v>
-      </c>
-      <c r="O8" s="27">
-        <v>10</v>
-      </c>
-      <c r="P8" s="27">
-        <v>15</v>
-      </c>
-      <c r="Q8" s="15" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="9" spans="1:18" ht="15" x14ac:dyDescent="0.25">
-      <c r="A9" s="17" t="s">
-        <v>31</v>
-      </c>
-      <c r="B9" s="18" t="s">
-        <v>32</v>
-      </c>
-      <c r="C9" s="17">
-        <v>125674</v>
-      </c>
-      <c r="D9" s="19">
-        <v>9</v>
-      </c>
-      <c r="E9" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="F9" s="20"/>
-      <c r="G9" s="20"/>
-      <c r="H9" s="25">
-        <v>0</v>
-      </c>
-      <c r="I9" s="23">
-        <v>13</v>
-      </c>
-      <c r="J9" s="23">
-        <v>55</v>
-      </c>
-      <c r="K9" s="23" t="s">
-        <v>14</v>
-      </c>
-      <c r="L9" s="23" t="s">
-        <v>14</v>
-      </c>
-      <c r="M9" s="23" t="s">
-        <v>14</v>
-      </c>
-      <c r="N9" s="23" t="s">
-        <v>14</v>
-      </c>
-      <c r="O9" s="23" t="s">
-        <v>14</v>
-      </c>
-      <c r="P9" s="23" t="s">
-        <v>14</v>
-      </c>
-      <c r="Q9" s="21" t="s">
-        <v>38</v>
-      </c>
+      <c r="F9" s="12"/>
+      <c r="G9" s="12"/>
+      <c r="H9" s="24">
+        <v>0</v>
+      </c>
+      <c r="I9" s="22">
+        <v>0</v>
+      </c>
+      <c r="J9" s="22">
+        <v>23.15</v>
+      </c>
+      <c r="K9" s="22">
+        <v>5</v>
+      </c>
+      <c r="L9" s="22">
+        <v>23.15</v>
+      </c>
+      <c r="M9" s="26">
+        <v>5</v>
+      </c>
+      <c r="N9" s="26">
+        <v>43.15</v>
+      </c>
+      <c r="O9" s="26">
+        <v>6</v>
+      </c>
+      <c r="P9" s="26">
+        <v>50.15</v>
+      </c>
+      <c r="Q9" s="13"/>
     </row>
     <row r="10" spans="1:18" ht="15" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C10" s="9">
-        <v>119789</v>
+        <v>115936</v>
       </c>
       <c r="D10" s="11">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F10" s="12"/>
       <c r="G10" s="12"/>
       <c r="H10" s="24">
         <v>0</v>
       </c>
-      <c r="I10" s="27"/>
-      <c r="J10" s="22"/>
-      <c r="K10" s="22"/>
-      <c r="L10" s="22"/>
-      <c r="M10" s="22"/>
-      <c r="N10" s="22"/>
+      <c r="I10" s="22">
+        <v>20</v>
+      </c>
+      <c r="J10" s="22">
+        <v>0</v>
+      </c>
+      <c r="K10" s="22">
+        <v>20</v>
+      </c>
+      <c r="L10" s="22">
+        <v>15</v>
+      </c>
+      <c r="M10" s="22">
+        <v>20</v>
+      </c>
+      <c r="N10" s="22">
+        <v>15</v>
+      </c>
       <c r="O10" s="22">
-        <v>5.15</v>
+        <v>35</v>
       </c>
       <c r="P10" s="22">
-        <v>28</v>
-      </c>
-      <c r="Q10" s="13"/>
+        <v>0</v>
+      </c>
+      <c r="Q10" s="13" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="11" spans="1:18" ht="15" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C11" s="9">
-        <v>120451</v>
+        <v>119789</v>
       </c>
       <c r="D11" s="11">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="F11" s="12"/>
       <c r="G11" s="12"/>
       <c r="H11" s="24">
         <v>0</v>
       </c>
-      <c r="I11" s="27"/>
+      <c r="I11" s="22"/>
       <c r="J11" s="22"/>
       <c r="K11" s="22"/>
       <c r="L11" s="22"/>
       <c r="M11" s="22"/>
       <c r="N11" s="22"/>
-      <c r="O11" s="26">
-        <v>19</v>
-      </c>
-      <c r="P11" s="26">
-        <v>22.5</v>
+      <c r="O11" s="22">
+        <v>5.15</v>
+      </c>
+      <c r="P11" s="22">
+        <v>28</v>
       </c>
       <c r="Q11" s="13"/>
     </row>
@@ -1793,6 +1800,9 @@
       <c r="H45" s="16"/>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:R11">
+    <sortCondition ref="A2:A11"/>
+  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup fitToHeight="0" orientation="landscape" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
@@ -1813,9 +1823,7 @@
     <col min="5" max="5" width="6.140625" style="1" customWidth="1"/>
     <col min="6" max="6" width="11.42578125" style="2" customWidth="1"/>
     <col min="7" max="7" width="10.28515625" style="2" customWidth="1"/>
-    <col min="8" max="8" width="12" customWidth="1"/>
-    <col min="9" max="9" width="12" style="28" customWidth="1"/>
-    <col min="10" max="14" width="12" customWidth="1"/>
+    <col min="8" max="14" width="12" customWidth="1"/>
     <col min="15" max="15" width="32.28515625" style="2" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1845,19 +1853,19 @@
         <v>7</v>
       </c>
       <c r="I1" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="J1" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="K1" s="7" t="s">
         <v>45</v>
-      </c>
-      <c r="J1" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="K1" s="7" t="s">
-        <v>46</v>
       </c>
       <c r="L1" s="7" t="s">
         <v>8</v>
       </c>
       <c r="M1" s="7" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="N1" s="7" t="s">
         <v>9</v>
@@ -1867,343 +1875,141 @@
       </c>
     </row>
     <row r="2" spans="1:16" ht="15" x14ac:dyDescent="0.25">
-      <c r="A2" s="9" t="s">
-        <v>21</v>
-      </c>
-      <c r="B2" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="C2" s="9">
-        <v>117031</v>
-      </c>
-      <c r="D2" s="11">
-        <v>10</v>
-      </c>
-      <c r="E2" s="10" t="s">
-        <v>16</v>
-      </c>
+      <c r="A2" s="9"/>
+      <c r="B2" s="10"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="10"/>
       <c r="F2" s="12"/>
       <c r="G2" s="12"/>
-      <c r="H2" s="24">
-        <v>0</v>
-      </c>
-      <c r="I2" s="26">
-        <v>0</v>
-      </c>
-      <c r="J2" s="26">
-        <v>40</v>
-      </c>
-      <c r="K2" s="26">
-        <v>6</v>
-      </c>
-      <c r="L2" s="26">
-        <v>40</v>
-      </c>
-      <c r="M2" s="26">
-        <v>6</v>
-      </c>
-      <c r="N2" s="26">
-        <v>52</v>
-      </c>
-      <c r="O2" s="13" t="s">
-        <v>34</v>
-      </c>
+      <c r="H2" s="24"/>
+      <c r="I2" s="22"/>
+      <c r="J2" s="22"/>
+      <c r="K2" s="22"/>
+      <c r="L2" s="22"/>
+      <c r="M2" s="22"/>
+      <c r="N2" s="22"/>
+      <c r="O2" s="13"/>
     </row>
     <row r="3" spans="1:16" ht="15" x14ac:dyDescent="0.25">
-      <c r="A3" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="B3" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="C3" s="9">
-        <v>116157</v>
-      </c>
-      <c r="D3" s="11">
-        <v>12</v>
-      </c>
-      <c r="E3" s="10" t="s">
-        <v>15</v>
-      </c>
+      <c r="A3" s="9"/>
+      <c r="B3" s="10"/>
+      <c r="C3" s="9"/>
+      <c r="D3" s="11"/>
+      <c r="E3" s="10"/>
       <c r="F3" s="12"/>
       <c r="G3" s="12"/>
-      <c r="H3" s="24">
-        <v>0</v>
-      </c>
-      <c r="I3" s="27">
-        <v>0</v>
-      </c>
-      <c r="J3" s="27">
-        <v>23.15</v>
-      </c>
-      <c r="K3" s="27">
-        <v>5</v>
-      </c>
-      <c r="L3" s="27">
-        <v>23.15</v>
-      </c>
-      <c r="M3" s="26">
-        <v>5</v>
-      </c>
-      <c r="N3" s="26">
-        <v>43.15</v>
-      </c>
+      <c r="H3" s="24"/>
+      <c r="I3" s="22"/>
+      <c r="J3" s="22"/>
+      <c r="K3" s="22"/>
+      <c r="L3" s="22"/>
+      <c r="M3" s="22"/>
+      <c r="N3" s="22"/>
       <c r="O3" s="13"/>
     </row>
     <row r="4" spans="1:16" ht="15" x14ac:dyDescent="0.25">
-      <c r="A4" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="B4" s="10" t="s">
-        <v>18</v>
-      </c>
-      <c r="C4" s="9">
-        <v>115936</v>
-      </c>
-      <c r="D4" s="11">
-        <v>8</v>
-      </c>
-      <c r="E4" s="10" t="s">
-        <v>13</v>
-      </c>
+      <c r="A4" s="9"/>
+      <c r="B4" s="10"/>
+      <c r="C4" s="9"/>
+      <c r="D4" s="11"/>
+      <c r="E4" s="10"/>
       <c r="F4" s="12"/>
       <c r="G4" s="12"/>
-      <c r="H4" s="24">
-        <v>0</v>
-      </c>
-      <c r="I4" s="27">
-        <v>20</v>
-      </c>
-      <c r="J4" s="27">
-        <v>0</v>
-      </c>
-      <c r="K4" s="27">
-        <v>20</v>
-      </c>
-      <c r="L4" s="27">
-        <v>15</v>
-      </c>
-      <c r="M4" s="27">
-        <v>20</v>
-      </c>
-      <c r="N4" s="27">
-        <v>15</v>
-      </c>
-      <c r="O4" s="13" t="s">
-        <v>35</v>
-      </c>
+      <c r="H4" s="24"/>
+      <c r="I4" s="22"/>
+      <c r="J4" s="22"/>
+      <c r="K4" s="22"/>
+      <c r="L4" s="22"/>
+      <c r="M4" s="22"/>
+      <c r="N4" s="22"/>
+      <c r="O4" s="13"/>
     </row>
     <row r="5" spans="1:16" ht="15" x14ac:dyDescent="0.25">
-      <c r="A5" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="B5" s="10" t="s">
-        <v>24</v>
-      </c>
-      <c r="C5" s="9">
-        <v>118245</v>
-      </c>
-      <c r="D5" s="11">
-        <v>7</v>
-      </c>
-      <c r="E5" s="10" t="s">
-        <v>11</v>
-      </c>
+      <c r="A5" s="9"/>
+      <c r="B5" s="10"/>
+      <c r="C5" s="9"/>
+      <c r="D5" s="11"/>
+      <c r="E5" s="10"/>
       <c r="F5" s="12"/>
       <c r="G5" s="12"/>
-      <c r="H5" s="24">
-        <v>0</v>
-      </c>
-      <c r="I5" s="27">
-        <v>0</v>
-      </c>
-      <c r="J5" s="27"/>
-      <c r="K5" s="27">
-        <v>15</v>
-      </c>
-      <c r="L5" s="27">
-        <v>0</v>
-      </c>
-      <c r="M5" s="27">
-        <v>15</v>
-      </c>
-      <c r="N5" s="27">
-        <v>0</v>
-      </c>
+      <c r="H5" s="24"/>
+      <c r="I5" s="22"/>
+      <c r="J5" s="22"/>
+      <c r="K5" s="22"/>
+      <c r="L5" s="22"/>
+      <c r="M5" s="22"/>
+      <c r="N5" s="22"/>
       <c r="O5" s="13"/>
     </row>
     <row r="6" spans="1:16" ht="15" x14ac:dyDescent="0.25">
-      <c r="A6" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="B6" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="C6" s="9">
-        <v>118678</v>
-      </c>
-      <c r="D6" s="11">
-        <v>9</v>
-      </c>
-      <c r="E6" s="10" t="s">
-        <v>16</v>
-      </c>
+      <c r="A6" s="9"/>
+      <c r="B6" s="10"/>
+      <c r="C6" s="9"/>
+      <c r="D6" s="11"/>
+      <c r="E6" s="10"/>
       <c r="F6" s="12"/>
       <c r="G6" s="12"/>
-      <c r="H6" s="24">
-        <v>0</v>
-      </c>
-      <c r="I6" s="27">
-        <v>0</v>
-      </c>
-      <c r="J6" s="27">
-        <v>0</v>
-      </c>
-      <c r="K6" s="27">
-        <v>0</v>
-      </c>
-      <c r="L6" s="27">
-        <v>10</v>
-      </c>
-      <c r="M6" s="27">
-        <v>0</v>
-      </c>
-      <c r="N6" s="27">
-        <v>10</v>
-      </c>
+      <c r="H6" s="24"/>
+      <c r="I6" s="22"/>
+      <c r="J6" s="22"/>
+      <c r="K6" s="22"/>
+      <c r="L6" s="22"/>
+      <c r="M6" s="22"/>
+      <c r="N6" s="22"/>
       <c r="O6" s="13"/>
     </row>
     <row r="7" spans="1:16" ht="15" x14ac:dyDescent="0.25">
-      <c r="A7" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="B7" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="C7" s="9">
-        <v>121874</v>
-      </c>
-      <c r="D7" s="11">
-        <v>8</v>
-      </c>
-      <c r="E7" s="10" t="s">
-        <v>13</v>
-      </c>
+      <c r="A7" s="9"/>
+      <c r="B7" s="10"/>
+      <c r="C7" s="9"/>
+      <c r="D7" s="11"/>
+      <c r="E7" s="10"/>
       <c r="F7" s="12"/>
       <c r="G7" s="12"/>
-      <c r="H7" s="24">
-        <v>8.25</v>
-      </c>
-      <c r="I7" s="26">
-        <v>42.33</v>
-      </c>
-      <c r="J7" s="26">
-        <v>14</v>
-      </c>
-      <c r="K7" s="26">
-        <v>42.33</v>
-      </c>
-      <c r="L7" s="26">
-        <v>14</v>
-      </c>
-      <c r="M7" s="26">
-        <v>42.33</v>
-      </c>
-      <c r="N7" s="26">
-        <v>32</v>
-      </c>
-      <c r="O7" s="13" t="s">
-        <v>36</v>
-      </c>
-      <c r="P7" s="14" t="s">
-        <v>33</v>
-      </c>
+      <c r="H7" s="24"/>
+      <c r="I7" s="22"/>
+      <c r="J7" s="22"/>
+      <c r="K7" s="22"/>
+      <c r="L7" s="22"/>
+      <c r="M7" s="22"/>
+      <c r="N7" s="22"/>
+      <c r="O7" s="13"/>
+      <c r="P7" s="14"/>
     </row>
     <row r="8" spans="1:16" ht="15" x14ac:dyDescent="0.25">
-      <c r="A8" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="B8" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="C8" s="9">
-        <v>122965</v>
-      </c>
-      <c r="D8" s="11">
-        <v>7</v>
-      </c>
-      <c r="E8" s="10" t="s">
-        <v>11</v>
-      </c>
+      <c r="A8" s="9"/>
+      <c r="B8" s="10"/>
+      <c r="C8" s="9"/>
+      <c r="D8" s="11"/>
+      <c r="E8" s="10"/>
       <c r="F8" s="12"/>
       <c r="G8" s="12"/>
-      <c r="H8" s="24">
-        <v>0</v>
-      </c>
-      <c r="I8" s="27">
-        <v>10</v>
-      </c>
-      <c r="J8" s="27">
-        <v>15</v>
-      </c>
-      <c r="K8" s="27">
-        <v>10</v>
-      </c>
-      <c r="L8" s="27">
-        <v>15</v>
-      </c>
-      <c r="M8" s="26">
-        <v>10</v>
-      </c>
-      <c r="N8" s="26">
-        <v>34</v>
-      </c>
-      <c r="O8" s="15" t="s">
-        <v>37</v>
-      </c>
+      <c r="H8" s="24"/>
+      <c r="I8" s="22"/>
+      <c r="J8" s="22"/>
+      <c r="K8" s="22"/>
+      <c r="L8" s="22"/>
+      <c r="M8" s="22"/>
+      <c r="N8" s="22"/>
+      <c r="O8" s="15"/>
     </row>
     <row r="9" spans="1:16" ht="15" x14ac:dyDescent="0.25">
-      <c r="A9" s="17" t="s">
-        <v>31</v>
-      </c>
-      <c r="B9" s="18" t="s">
-        <v>32</v>
-      </c>
-      <c r="C9" s="17">
-        <v>125674</v>
-      </c>
-      <c r="D9" s="19">
-        <v>9</v>
-      </c>
-      <c r="E9" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="F9" s="20"/>
-      <c r="G9" s="20"/>
-      <c r="H9" s="25">
-        <v>0</v>
-      </c>
-      <c r="I9" s="23">
-        <v>13</v>
-      </c>
-      <c r="J9" s="23">
-        <v>55</v>
-      </c>
-      <c r="K9" s="23" t="s">
-        <v>14</v>
-      </c>
-      <c r="L9" s="23" t="s">
-        <v>14</v>
-      </c>
-      <c r="M9" s="23" t="s">
-        <v>14</v>
-      </c>
-      <c r="N9" s="23" t="s">
-        <v>14</v>
-      </c>
-      <c r="O9" s="21" t="s">
-        <v>38</v>
-      </c>
+      <c r="A9" s="9"/>
+      <c r="B9" s="10"/>
+      <c r="C9" s="9"/>
+      <c r="D9" s="11"/>
+      <c r="E9" s="10"/>
+      <c r="F9" s="12"/>
+      <c r="G9" s="12"/>
+      <c r="H9" s="28"/>
+      <c r="I9" s="22"/>
+      <c r="J9" s="22"/>
+      <c r="K9" s="22"/>
+      <c r="L9" s="22"/>
+      <c r="M9" s="22"/>
+      <c r="N9" s="22"/>
+      <c r="O9" s="27"/>
     </row>
     <row r="10" spans="1:16" ht="15" x14ac:dyDescent="0.25">
       <c r="A10" s="9"/>
@@ -2214,7 +2020,7 @@
       <c r="F10" s="12"/>
       <c r="G10" s="12"/>
       <c r="H10" s="24"/>
-      <c r="I10" s="27"/>
+      <c r="I10" s="22"/>
       <c r="J10" s="22"/>
       <c r="K10" s="22"/>
       <c r="L10" s="22"/>
@@ -2231,7 +2037,7 @@
       <c r="F11" s="12"/>
       <c r="G11" s="12"/>
       <c r="H11" s="24"/>
-      <c r="I11" s="27"/>
+      <c r="I11" s="22"/>
       <c r="J11" s="22"/>
       <c r="K11" s="22"/>
       <c r="L11" s="22"/>

</xml_diff>

<commit_message>
Added missing columns to sheet and added letter status to status report
</commit_message>
<xml_diff>
--- a/Testing/basic_sequence/workbook.xlsx
+++ b/Testing/basic_sequence/workbook.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Pavan Rauch\git\Truancy-Local\Testing\basic_sequence\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BF430B2-4C74-47B1-893B-EB530D8C29F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{098948B8-56D6-45A8-8784-CC0EE9BD252B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Urbana Elementary (Before)" sheetId="4" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="53">
   <si>
     <t>Last Name</t>
   </si>
@@ -174,6 +174,18 @@
   </si>
   <si>
     <t>Doe</t>
+  </si>
+  <si>
+    <t>Phone/Email</t>
+  </si>
+  <si>
+    <t>Date Preliminary Letter Sent</t>
+  </si>
+  <si>
+    <t>Date Mediation Letter Sent</t>
+  </si>
+  <si>
+    <t>Mediation Date/Time</t>
   </si>
 </sst>
 </file>
@@ -183,7 +195,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -212,6 +224,13 @@
       <family val="2"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -283,7 +302,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -359,6 +378,10 @@
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -623,7 +646,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P45"/>
+  <dimension ref="A1:T45"/>
   <sheetFormatPr defaultColWidth="8.28515625" defaultRowHeight="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.5703125" customWidth="1"/>
@@ -631,13 +654,14 @@
     <col min="3" max="3" width="9.85546875" customWidth="1"/>
     <col min="4" max="4" width="6" customWidth="1"/>
     <col min="5" max="5" width="6.140625" style="1" customWidth="1"/>
-    <col min="6" max="6" width="11.42578125" style="2" customWidth="1"/>
-    <col min="7" max="7" width="10.28515625" style="2" customWidth="1"/>
-    <col min="8" max="14" width="12" customWidth="1"/>
-    <col min="15" max="15" width="32.28515625" style="2" customWidth="1"/>
+    <col min="6" max="7" width="11.42578125" style="2" customWidth="1"/>
+    <col min="8" max="8" width="13.5703125" style="2" customWidth="1"/>
+    <col min="9" max="15" width="12" customWidth="1"/>
+    <col min="16" max="16" width="32.28515625" style="2" customWidth="1"/>
+    <col min="17" max="19" width="16.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="45" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:20" ht="45" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -659,32 +683,44 @@
       <c r="G1" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="H1" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="I1" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="7" t="s">
+      <c r="J1" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="J1" s="7" t="s">
+      <c r="K1" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="K1" s="7" t="s">
+      <c r="L1" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="L1" s="7" t="s">
+      <c r="M1" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="M1" s="7" t="s">
+      <c r="N1" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="N1" s="7" t="s">
+      <c r="O1" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="O1" s="8" t="s">
+      <c r="P1" s="8" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="2" spans="1:16" ht="15" x14ac:dyDescent="0.25">
+      <c r="Q1" s="29" t="s">
+        <v>50</v>
+      </c>
+      <c r="R1" s="29" t="s">
+        <v>51</v>
+      </c>
+      <c r="S1" s="29" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="2" spans="1:20" ht="15" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
         <v>24</v>
       </c>
@@ -702,10 +738,8 @@
       </c>
       <c r="F2" s="12"/>
       <c r="G2" s="12"/>
-      <c r="H2" s="24">
-        <v>0</v>
-      </c>
-      <c r="I2" s="22">
+      <c r="H2" s="12"/>
+      <c r="I2" s="24">
         <v>0</v>
       </c>
       <c r="J2" s="22">
@@ -715,17 +749,20 @@
         <v>0</v>
       </c>
       <c r="L2" s="22">
+        <v>0</v>
+      </c>
+      <c r="M2" s="22">
         <v>10</v>
       </c>
-      <c r="M2" s="22">
-        <v>0</v>
-      </c>
       <c r="N2" s="22">
+        <v>0</v>
+      </c>
+      <c r="O2" s="22">
         <v>10</v>
       </c>
-      <c r="O2" s="13"/>
-    </row>
-    <row r="3" spans="1:16" ht="15" x14ac:dyDescent="0.25">
+      <c r="P2" s="13"/>
+    </row>
+    <row r="3" spans="1:20" ht="15" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>22</v>
       </c>
@@ -743,28 +780,29 @@
       </c>
       <c r="F3" s="12"/>
       <c r="G3" s="12"/>
-      <c r="H3" s="24">
-        <v>0</v>
-      </c>
-      <c r="I3" s="22">
-        <v>0</v>
-      </c>
-      <c r="J3" s="22"/>
-      <c r="K3" s="22">
+      <c r="H3" s="12"/>
+      <c r="I3" s="24">
+        <v>0</v>
+      </c>
+      <c r="J3" s="22">
+        <v>0</v>
+      </c>
+      <c r="K3" s="22"/>
+      <c r="L3" s="22">
         <v>15</v>
       </c>
-      <c r="L3" s="22">
-        <v>0</v>
-      </c>
       <c r="M3" s="22">
+        <v>0</v>
+      </c>
+      <c r="N3" s="22">
         <v>15</v>
       </c>
-      <c r="N3" s="22">
-        <v>0</v>
-      </c>
-      <c r="O3" s="13"/>
-    </row>
-    <row r="4" spans="1:16" ht="15" x14ac:dyDescent="0.25">
+      <c r="O3" s="22">
+        <v>0</v>
+      </c>
+      <c r="P3" s="13"/>
+    </row>
+    <row r="4" spans="1:20" ht="15" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
         <v>20</v>
       </c>
@@ -782,32 +820,36 @@
       </c>
       <c r="F4" s="12"/>
       <c r="G4" s="12"/>
-      <c r="H4" s="24">
-        <v>0</v>
-      </c>
-      <c r="I4" s="26">
+      <c r="H4" s="12"/>
+      <c r="I4" s="24">
         <v>0</v>
       </c>
       <c r="J4" s="26">
+        <v>0</v>
+      </c>
+      <c r="K4" s="26">
         <v>40</v>
       </c>
-      <c r="K4" s="26">
+      <c r="L4" s="26">
         <v>6</v>
       </c>
-      <c r="L4" s="26">
+      <c r="M4" s="26">
         <v>40</v>
       </c>
-      <c r="M4" s="26">
+      <c r="N4" s="26">
         <v>6</v>
       </c>
-      <c r="N4" s="26">
+      <c r="O4" s="26">
         <v>52</v>
       </c>
-      <c r="O4" s="13" t="s">
+      <c r="P4" s="13" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="5" spans="1:16" ht="15" x14ac:dyDescent="0.25">
+      <c r="Q4" s="30">
+        <v>45672</v>
+      </c>
+    </row>
+    <row r="5" spans="1:20" ht="15" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
         <v>28</v>
       </c>
@@ -825,32 +867,33 @@
       </c>
       <c r="F5" s="12"/>
       <c r="G5" s="12"/>
-      <c r="H5" s="24">
-        <v>0</v>
-      </c>
-      <c r="I5" s="22">
+      <c r="H5" s="12"/>
+      <c r="I5" s="24">
+        <v>0</v>
+      </c>
+      <c r="J5" s="22">
         <v>10</v>
       </c>
-      <c r="J5" s="22">
+      <c r="K5" s="22">
         <v>15</v>
       </c>
-      <c r="K5" s="22">
+      <c r="L5" s="22">
         <v>10</v>
       </c>
-      <c r="L5" s="22">
+      <c r="M5" s="22">
         <v>15</v>
       </c>
-      <c r="M5" s="26">
+      <c r="N5" s="26">
         <v>10</v>
       </c>
-      <c r="N5" s="26">
+      <c r="O5" s="26">
         <v>34</v>
       </c>
-      <c r="O5" s="15" t="s">
+      <c r="P5" s="15" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="6" spans="1:16" ht="15" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:20" ht="15" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
         <v>26</v>
       </c>
@@ -868,35 +911,42 @@
       </c>
       <c r="F6" s="12"/>
       <c r="G6" s="12"/>
-      <c r="H6" s="24">
+      <c r="H6" s="12"/>
+      <c r="I6" s="24">
         <v>8.25</v>
       </c>
-      <c r="I6" s="26">
+      <c r="J6" s="26">
         <v>42.33</v>
       </c>
-      <c r="J6" s="26">
+      <c r="K6" s="26">
         <v>14</v>
       </c>
-      <c r="K6" s="26">
+      <c r="L6" s="26">
         <v>42.33</v>
       </c>
-      <c r="L6" s="26">
+      <c r="M6" s="26">
         <v>14</v>
       </c>
-      <c r="M6" s="26">
+      <c r="N6" s="26">
         <v>42.33</v>
       </c>
-      <c r="N6" s="26">
+      <c r="O6" s="26">
         <v>32</v>
       </c>
-      <c r="O6" s="13" t="s">
+      <c r="P6" s="13" t="s">
         <v>35</v>
       </c>
-      <c r="P6" s="14" t="s">
+      <c r="Q6" s="30">
+        <v>45664</v>
+      </c>
+      <c r="R6" s="30">
+        <v>45680</v>
+      </c>
+      <c r="T6" s="14" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="7" spans="1:16" ht="15" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:20" ht="15" x14ac:dyDescent="0.25">
       <c r="A7" s="17" t="s">
         <v>30</v>
       </c>
@@ -914,17 +964,15 @@
       </c>
       <c r="F7" s="20"/>
       <c r="G7" s="20"/>
-      <c r="H7" s="25">
-        <v>0</v>
-      </c>
-      <c r="I7" s="23">
+      <c r="H7" s="20"/>
+      <c r="I7" s="25">
+        <v>0</v>
+      </c>
+      <c r="J7" s="23">
         <v>13</v>
       </c>
-      <c r="J7" s="23">
+      <c r="K7" s="23">
         <v>55</v>
-      </c>
-      <c r="K7" s="23" t="s">
-        <v>14</v>
       </c>
       <c r="L7" s="23" t="s">
         <v>14</v>
@@ -935,11 +983,14 @@
       <c r="N7" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="O7" s="21" t="s">
+      <c r="O7" s="23" t="s">
+        <v>14</v>
+      </c>
+      <c r="P7" s="21" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="8" spans="1:16" ht="15" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:20" ht="15" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
         <v>18</v>
       </c>
@@ -957,30 +1008,31 @@
       </c>
       <c r="F8" s="12"/>
       <c r="G8" s="12"/>
-      <c r="H8" s="24">
-        <v>0</v>
-      </c>
-      <c r="I8" s="22">
+      <c r="H8" s="12"/>
+      <c r="I8" s="24">
         <v>0</v>
       </c>
       <c r="J8" s="22">
+        <v>0</v>
+      </c>
+      <c r="K8" s="22">
         <v>23.15</v>
       </c>
-      <c r="K8" s="22">
+      <c r="L8" s="22">
         <v>5</v>
       </c>
-      <c r="L8" s="22">
+      <c r="M8" s="22">
         <v>23.15</v>
       </c>
-      <c r="M8" s="26">
+      <c r="N8" s="26">
         <v>5</v>
       </c>
-      <c r="N8" s="26">
+      <c r="O8" s="26">
         <v>43.15</v>
       </c>
-      <c r="O8" s="13"/>
-    </row>
-    <row r="9" spans="1:16" ht="15" x14ac:dyDescent="0.25">
+      <c r="P8" s="13"/>
+    </row>
+    <row r="9" spans="1:20" ht="15" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
         <v>42</v>
       </c>
@@ -998,32 +1050,33 @@
       </c>
       <c r="F9" s="12"/>
       <c r="G9" s="12"/>
-      <c r="H9" s="24">
-        <v>0</v>
-      </c>
-      <c r="I9" s="22">
+      <c r="H9" s="12"/>
+      <c r="I9" s="24">
+        <v>0</v>
+      </c>
+      <c r="J9" s="22">
         <v>20</v>
       </c>
-      <c r="J9" s="22">
-        <v>0</v>
-      </c>
       <c r="K9" s="22">
+        <v>0</v>
+      </c>
+      <c r="L9" s="22">
         <v>20</v>
       </c>
-      <c r="L9" s="22">
+      <c r="M9" s="22">
         <v>15</v>
       </c>
-      <c r="M9" s="22">
+      <c r="N9" s="22">
         <v>20</v>
       </c>
-      <c r="N9" s="22">
+      <c r="O9" s="22">
         <v>15</v>
       </c>
-      <c r="O9" s="13" t="s">
+      <c r="P9" s="13" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="10" spans="1:16" ht="15" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:20" ht="15" x14ac:dyDescent="0.25">
       <c r="A10" s="9"/>
       <c r="B10" s="10"/>
       <c r="C10" s="9"/>
@@ -1031,16 +1084,17 @@
       <c r="E10" s="10"/>
       <c r="F10" s="12"/>
       <c r="G10" s="12"/>
-      <c r="H10" s="24"/>
-      <c r="I10" s="22"/>
+      <c r="H10" s="12"/>
+      <c r="I10" s="24"/>
       <c r="J10" s="22"/>
       <c r="K10" s="22"/>
       <c r="L10" s="22"/>
       <c r="M10" s="22"/>
       <c r="N10" s="22"/>
-      <c r="O10" s="13"/>
-    </row>
-    <row r="11" spans="1:16" ht="15" x14ac:dyDescent="0.25">
+      <c r="O10" s="22"/>
+      <c r="P10" s="13"/>
+    </row>
+    <row r="11" spans="1:20" ht="15" x14ac:dyDescent="0.25">
       <c r="A11" s="9"/>
       <c r="B11" s="10"/>
       <c r="C11" s="9"/>
@@ -1048,123 +1102,124 @@
       <c r="E11" s="10"/>
       <c r="F11" s="12"/>
       <c r="G11" s="12"/>
-      <c r="H11" s="24"/>
-      <c r="I11" s="22"/>
+      <c r="H11" s="12"/>
+      <c r="I11" s="24"/>
       <c r="J11" s="22"/>
       <c r="K11" s="22"/>
       <c r="L11" s="22"/>
       <c r="M11" s="22"/>
       <c r="N11" s="22"/>
-      <c r="O11" s="13"/>
-    </row>
-    <row r="12" spans="1:16" ht="15" x14ac:dyDescent="0.25">
-      <c r="H12" s="16"/>
-    </row>
-    <row r="13" spans="1:16" ht="15" x14ac:dyDescent="0.25">
-      <c r="H13" s="16"/>
-    </row>
-    <row r="14" spans="1:16" ht="15" x14ac:dyDescent="0.25">
-      <c r="H14" s="16"/>
-    </row>
-    <row r="15" spans="1:16" ht="15" x14ac:dyDescent="0.25">
-      <c r="H15" s="16"/>
-    </row>
-    <row r="16" spans="1:16" ht="15" x14ac:dyDescent="0.25">
-      <c r="H16" s="16"/>
-    </row>
-    <row r="17" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H17" s="16"/>
-    </row>
-    <row r="18" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H18" s="16"/>
-    </row>
-    <row r="19" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H19" s="16"/>
-    </row>
-    <row r="20" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H20" s="16"/>
-    </row>
-    <row r="21" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H21" s="16"/>
-    </row>
-    <row r="22" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H22" s="16"/>
-    </row>
-    <row r="23" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H23" s="16"/>
-    </row>
-    <row r="24" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H24" s="16"/>
-    </row>
-    <row r="25" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H25" s="16"/>
-    </row>
-    <row r="26" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H26" s="16"/>
-    </row>
-    <row r="27" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H27" s="16"/>
-    </row>
-    <row r="28" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H28" s="16"/>
-    </row>
-    <row r="29" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H29" s="16"/>
-    </row>
-    <row r="30" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H30" s="16"/>
-    </row>
-    <row r="31" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H31" s="16"/>
-    </row>
-    <row r="32" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H32" s="16"/>
-    </row>
-    <row r="33" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H33" s="16"/>
-    </row>
-    <row r="34" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H34" s="16"/>
-    </row>
-    <row r="35" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H35" s="16"/>
-    </row>
-    <row r="36" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H36" s="16"/>
-    </row>
-    <row r="37" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H37" s="16"/>
-    </row>
-    <row r="38" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H38" s="16"/>
-    </row>
-    <row r="39" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H39" s="16"/>
-    </row>
-    <row r="40" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H40" s="16"/>
-    </row>
-    <row r="41" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H41" s="16"/>
-    </row>
-    <row r="42" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H42" s="16"/>
-    </row>
-    <row r="43" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H43" s="16"/>
-    </row>
-    <row r="44" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H44" s="16"/>
-    </row>
-    <row r="45" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H45" s="16"/>
+      <c r="O11" s="22"/>
+      <c r="P11" s="13"/>
+    </row>
+    <row r="12" spans="1:20" ht="15" x14ac:dyDescent="0.25">
+      <c r="I12" s="16"/>
+    </row>
+    <row r="13" spans="1:20" ht="15" x14ac:dyDescent="0.25">
+      <c r="I13" s="16"/>
+    </row>
+    <row r="14" spans="1:20" ht="15" x14ac:dyDescent="0.25">
+      <c r="I14" s="16"/>
+    </row>
+    <row r="15" spans="1:20" ht="15" x14ac:dyDescent="0.25">
+      <c r="I15" s="16"/>
+    </row>
+    <row r="16" spans="1:20" ht="15" x14ac:dyDescent="0.25">
+      <c r="I16" s="16"/>
+    </row>
+    <row r="17" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I17" s="16"/>
+    </row>
+    <row r="18" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I18" s="16"/>
+    </row>
+    <row r="19" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I19" s="16"/>
+    </row>
+    <row r="20" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I20" s="16"/>
+    </row>
+    <row r="21" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I21" s="16"/>
+    </row>
+    <row r="22" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I22" s="16"/>
+    </row>
+    <row r="23" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I23" s="16"/>
+    </row>
+    <row r="24" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I24" s="16"/>
+    </row>
+    <row r="25" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I25" s="16"/>
+    </row>
+    <row r="26" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I26" s="16"/>
+    </row>
+    <row r="27" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I27" s="16"/>
+    </row>
+    <row r="28" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I28" s="16"/>
+    </row>
+    <row r="29" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I29" s="16"/>
+    </row>
+    <row r="30" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I30" s="16"/>
+    </row>
+    <row r="31" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I31" s="16"/>
+    </row>
+    <row r="32" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I32" s="16"/>
+    </row>
+    <row r="33" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I33" s="16"/>
+    </row>
+    <row r="34" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I34" s="16"/>
+    </row>
+    <row r="35" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I35" s="16"/>
+    </row>
+    <row r="36" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I36" s="16"/>
+    </row>
+    <row r="37" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I37" s="16"/>
+    </row>
+    <row r="38" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I38" s="16"/>
+    </row>
+    <row r="39" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I39" s="16"/>
+    </row>
+    <row r="40" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I40" s="16"/>
+    </row>
+    <row r="41" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I41" s="16"/>
+    </row>
+    <row r="42" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I42" s="16"/>
+    </row>
+    <row r="43" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I43" s="16"/>
+    </row>
+    <row r="44" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I44" s="16"/>
+    </row>
+    <row r="45" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I45" s="16"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:P9">
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:Q9">
     <sortCondition ref="A2:A9"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup fitToHeight="0" orientation="landscape" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup fitToHeight="0" orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1173,7 +1228,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:R45"/>
+  <dimension ref="A1:V45"/>
   <sheetFormatPr defaultColWidth="8.28515625" defaultRowHeight="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.5703125" customWidth="1"/>
@@ -1181,13 +1236,14 @@
     <col min="3" max="3" width="9.85546875" customWidth="1"/>
     <col min="4" max="4" width="6" customWidth="1"/>
     <col min="5" max="5" width="6.140625" style="1" customWidth="1"/>
-    <col min="6" max="6" width="11.42578125" style="2" customWidth="1"/>
-    <col min="7" max="7" width="10.28515625" style="2" customWidth="1"/>
-    <col min="8" max="16" width="12" customWidth="1"/>
-    <col min="17" max="17" width="32.28515625" style="2" customWidth="1"/>
+    <col min="6" max="7" width="11.42578125" style="2" customWidth="1"/>
+    <col min="8" max="8" width="13.5703125" style="2" customWidth="1"/>
+    <col min="9" max="17" width="12" customWidth="1"/>
+    <col min="18" max="18" width="32.28515625" style="2" customWidth="1"/>
+    <col min="19" max="21" width="16.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="45" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:22" ht="45" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1209,38 +1265,50 @@
       <c r="G1" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="H1" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="I1" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="7" t="s">
+      <c r="J1" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="J1" s="7" t="s">
+      <c r="K1" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="K1" s="7" t="s">
+      <c r="L1" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="L1" s="7" t="s">
+      <c r="M1" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="M1" s="7" t="s">
+      <c r="N1" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="N1" s="7" t="s">
+      <c r="O1" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="O1" s="7" t="s">
+      <c r="P1" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="P1" s="7" t="s">
+      <c r="Q1" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="Q1" s="8" t="s">
+      <c r="R1" s="8" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="2" spans="1:18" ht="15" x14ac:dyDescent="0.25">
+      <c r="S1" s="29" t="s">
+        <v>50</v>
+      </c>
+      <c r="T1" s="29" t="s">
+        <v>51</v>
+      </c>
+      <c r="U1" s="29" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="2" spans="1:22" ht="15" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
         <v>24</v>
       </c>
@@ -1258,10 +1326,8 @@
       </c>
       <c r="F2" s="12"/>
       <c r="G2" s="12"/>
-      <c r="H2" s="24">
-        <v>0</v>
-      </c>
-      <c r="I2" s="22">
+      <c r="H2" s="12"/>
+      <c r="I2" s="24">
         <v>0</v>
       </c>
       <c r="J2" s="22">
@@ -1271,23 +1337,26 @@
         <v>0</v>
       </c>
       <c r="L2" s="22">
+        <v>0</v>
+      </c>
+      <c r="M2" s="22">
         <v>10</v>
       </c>
-      <c r="M2" s="22">
-        <v>0</v>
-      </c>
       <c r="N2" s="22">
+        <v>0</v>
+      </c>
+      <c r="O2" s="22">
         <v>10</v>
       </c>
-      <c r="O2" s="22">
+      <c r="P2" s="22">
         <v>2</v>
       </c>
-      <c r="P2" s="22">
+      <c r="Q2" s="22">
         <v>10</v>
       </c>
-      <c r="Q2" s="13"/>
-    </row>
-    <row r="3" spans="1:18" ht="15" x14ac:dyDescent="0.25">
+      <c r="R2" s="13"/>
+    </row>
+    <row r="3" spans="1:22" ht="15" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>22</v>
       </c>
@@ -1305,34 +1374,35 @@
       </c>
       <c r="F3" s="12"/>
       <c r="G3" s="12"/>
-      <c r="H3" s="24">
-        <v>0</v>
-      </c>
-      <c r="I3" s="22">
-        <v>0</v>
-      </c>
-      <c r="J3" s="22"/>
-      <c r="K3" s="22">
+      <c r="H3" s="12"/>
+      <c r="I3" s="24">
+        <v>0</v>
+      </c>
+      <c r="J3" s="22">
+        <v>0</v>
+      </c>
+      <c r="K3" s="22"/>
+      <c r="L3" s="22">
         <v>15</v>
       </c>
-      <c r="L3" s="22">
-        <v>0</v>
-      </c>
       <c r="M3" s="22">
+        <v>0</v>
+      </c>
+      <c r="N3" s="22">
         <v>15</v>
       </c>
-      <c r="N3" s="22">
-        <v>0</v>
-      </c>
-      <c r="O3" s="26">
+      <c r="O3" s="22">
+        <v>0</v>
+      </c>
+      <c r="P3" s="26">
         <v>50</v>
       </c>
-      <c r="P3" s="26">
-        <v>0</v>
-      </c>
-      <c r="Q3" s="13"/>
-    </row>
-    <row r="4" spans="1:18" ht="15" x14ac:dyDescent="0.25">
+      <c r="Q3" s="26">
+        <v>0</v>
+      </c>
+      <c r="R3" s="13"/>
+    </row>
+    <row r="4" spans="1:22" ht="15" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
         <v>48</v>
       </c>
@@ -1350,24 +1420,25 @@
       </c>
       <c r="F4" s="12"/>
       <c r="G4" s="12"/>
-      <c r="H4" s="24">
-        <v>0</v>
-      </c>
-      <c r="I4" s="22"/>
+      <c r="H4" s="12"/>
+      <c r="I4" s="24">
+        <v>0</v>
+      </c>
       <c r="J4" s="22"/>
       <c r="K4" s="22"/>
       <c r="L4" s="22"/>
       <c r="M4" s="22"/>
       <c r="N4" s="22"/>
-      <c r="O4" s="26">
+      <c r="O4" s="22"/>
+      <c r="P4" s="26">
         <v>19</v>
       </c>
-      <c r="P4" s="26">
+      <c r="Q4" s="26">
         <v>22.5</v>
       </c>
-      <c r="Q4" s="13"/>
-    </row>
-    <row r="5" spans="1:18" ht="15" x14ac:dyDescent="0.25">
+      <c r="R4" s="13"/>
+    </row>
+    <row r="5" spans="1:22" ht="15" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
         <v>20</v>
       </c>
@@ -1385,38 +1456,39 @@
       </c>
       <c r="F5" s="12"/>
       <c r="G5" s="12"/>
-      <c r="H5" s="24">
+      <c r="H5" s="12"/>
+      <c r="I5" s="24">
         <v>19.399999999999999</v>
       </c>
-      <c r="I5" s="26">
-        <v>0</v>
-      </c>
       <c r="J5" s="26">
+        <v>0</v>
+      </c>
+      <c r="K5" s="26">
         <v>40</v>
       </c>
-      <c r="K5" s="26">
+      <c r="L5" s="26">
         <v>6</v>
       </c>
-      <c r="L5" s="26">
+      <c r="M5" s="26">
         <v>40</v>
       </c>
-      <c r="M5" s="26">
+      <c r="N5" s="26">
         <v>6</v>
       </c>
-      <c r="N5" s="26">
+      <c r="O5" s="26">
         <v>52</v>
       </c>
-      <c r="O5" s="26">
+      <c r="P5" s="26">
         <v>6</v>
       </c>
-      <c r="P5" s="26">
+      <c r="Q5" s="26">
         <v>62</v>
       </c>
-      <c r="Q5" s="13" t="s">
+      <c r="R5" s="13" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="6" spans="1:18" ht="15" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:22" ht="15" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
         <v>28</v>
       </c>
@@ -1434,38 +1506,39 @@
       </c>
       <c r="F6" s="12"/>
       <c r="G6" s="12"/>
-      <c r="H6" s="24">
-        <v>0</v>
-      </c>
-      <c r="I6" s="22">
+      <c r="H6" s="12"/>
+      <c r="I6" s="24">
+        <v>0</v>
+      </c>
+      <c r="J6" s="22">
         <v>10</v>
       </c>
-      <c r="J6" s="22">
+      <c r="K6" s="22">
         <v>15</v>
       </c>
-      <c r="K6" s="22">
+      <c r="L6" s="22">
         <v>10</v>
       </c>
-      <c r="L6" s="22">
+      <c r="M6" s="22">
         <v>15</v>
       </c>
-      <c r="M6" s="26">
+      <c r="N6" s="26">
         <v>10</v>
       </c>
-      <c r="N6" s="26">
+      <c r="O6" s="26">
         <v>34</v>
       </c>
-      <c r="O6" s="22">
+      <c r="P6" s="22">
         <v>10</v>
       </c>
-      <c r="P6" s="22">
+      <c r="Q6" s="22">
         <v>15</v>
       </c>
-      <c r="Q6" s="15" t="s">
+      <c r="R6" s="15" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="7" spans="1:18" ht="15" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:22" ht="15" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
         <v>26</v>
       </c>
@@ -1483,41 +1556,42 @@
       </c>
       <c r="F7" s="12"/>
       <c r="G7" s="12"/>
-      <c r="H7" s="24">
+      <c r="H7" s="12"/>
+      <c r="I7" s="24">
         <v>8.25</v>
       </c>
-      <c r="I7" s="26">
+      <c r="J7" s="26">
         <v>42.33</v>
       </c>
-      <c r="J7" s="26">
+      <c r="K7" s="26">
         <v>14</v>
       </c>
-      <c r="K7" s="26">
+      <c r="L7" s="26">
         <v>42.33</v>
       </c>
-      <c r="L7" s="26">
+      <c r="M7" s="26">
         <v>14</v>
       </c>
-      <c r="M7" s="26">
+      <c r="N7" s="26">
         <v>42.33</v>
       </c>
-      <c r="N7" s="26">
+      <c r="O7" s="26">
         <v>32</v>
-      </c>
-      <c r="O7" s="22" t="s">
-        <v>14</v>
       </c>
       <c r="P7" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="Q7" s="13" t="s">
+      <c r="Q7" s="22" t="s">
+        <v>14</v>
+      </c>
+      <c r="R7" s="13" t="s">
         <v>35</v>
       </c>
-      <c r="R7" s="14" t="s">
+      <c r="V7" s="14" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="8" spans="1:18" ht="15" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:22" ht="15" x14ac:dyDescent="0.25">
       <c r="A8" s="17" t="s">
         <v>30</v>
       </c>
@@ -1535,17 +1609,15 @@
       </c>
       <c r="F8" s="20"/>
       <c r="G8" s="20"/>
-      <c r="H8" s="25">
-        <v>0</v>
-      </c>
-      <c r="I8" s="23">
+      <c r="H8" s="20"/>
+      <c r="I8" s="25">
+        <v>0</v>
+      </c>
+      <c r="J8" s="23">
         <v>13</v>
       </c>
-      <c r="J8" s="23">
+      <c r="K8" s="23">
         <v>55</v>
-      </c>
-      <c r="K8" s="23" t="s">
-        <v>14</v>
       </c>
       <c r="L8" s="23" t="s">
         <v>14</v>
@@ -1562,11 +1634,14 @@
       <c r="P8" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="Q8" s="21" t="s">
+      <c r="Q8" s="23" t="s">
+        <v>14</v>
+      </c>
+      <c r="R8" s="21" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="9" spans="1:18" ht="15" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:22" ht="15" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
         <v>18</v>
       </c>
@@ -1584,36 +1659,37 @@
       </c>
       <c r="F9" s="12"/>
       <c r="G9" s="12"/>
-      <c r="H9" s="24">
-        <v>0</v>
-      </c>
-      <c r="I9" s="22">
+      <c r="H9" s="12"/>
+      <c r="I9" s="24">
         <v>0</v>
       </c>
       <c r="J9" s="22">
+        <v>0</v>
+      </c>
+      <c r="K9" s="22">
         <v>23.15</v>
       </c>
-      <c r="K9" s="22">
+      <c r="L9" s="22">
         <v>5</v>
       </c>
-      <c r="L9" s="22">
+      <c r="M9" s="22">
         <v>23.15</v>
       </c>
-      <c r="M9" s="26">
+      <c r="N9" s="26">
         <v>5</v>
       </c>
-      <c r="N9" s="26">
+      <c r="O9" s="26">
         <v>43.15</v>
       </c>
-      <c r="O9" s="26">
+      <c r="P9" s="26">
         <v>6</v>
       </c>
-      <c r="P9" s="26">
+      <c r="Q9" s="26">
         <v>50.15</v>
       </c>
-      <c r="Q9" s="13"/>
-    </row>
-    <row r="10" spans="1:18" ht="15" x14ac:dyDescent="0.25">
+      <c r="R9" s="13"/>
+    </row>
+    <row r="10" spans="1:22" ht="15" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
         <v>42</v>
       </c>
@@ -1631,38 +1707,39 @@
       </c>
       <c r="F10" s="12"/>
       <c r="G10" s="12"/>
-      <c r="H10" s="24">
-        <v>0</v>
-      </c>
-      <c r="I10" s="22">
+      <c r="H10" s="12"/>
+      <c r="I10" s="24">
+        <v>0</v>
+      </c>
+      <c r="J10" s="22">
         <v>20</v>
       </c>
-      <c r="J10" s="22">
-        <v>0</v>
-      </c>
       <c r="K10" s="22">
+        <v>0</v>
+      </c>
+      <c r="L10" s="22">
         <v>20</v>
       </c>
-      <c r="L10" s="22">
+      <c r="M10" s="22">
         <v>15</v>
       </c>
-      <c r="M10" s="22">
+      <c r="N10" s="22">
         <v>20</v>
       </c>
-      <c r="N10" s="22">
+      <c r="O10" s="22">
         <v>15</v>
       </c>
-      <c r="O10" s="22">
+      <c r="P10" s="22">
         <v>35</v>
       </c>
-      <c r="P10" s="22">
-        <v>0</v>
-      </c>
-      <c r="Q10" s="13" t="s">
+      <c r="Q10" s="22">
+        <v>0</v>
+      </c>
+      <c r="R10" s="13" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="11" spans="1:18" ht="15" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:22" ht="15" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
         <v>40</v>
       </c>
@@ -1680,127 +1757,128 @@
       </c>
       <c r="F11" s="12"/>
       <c r="G11" s="12"/>
-      <c r="H11" s="24">
-        <v>0</v>
-      </c>
-      <c r="I11" s="22"/>
+      <c r="H11" s="12"/>
+      <c r="I11" s="24">
+        <v>0</v>
+      </c>
       <c r="J11" s="22"/>
       <c r="K11" s="22"/>
       <c r="L11" s="22"/>
       <c r="M11" s="22"/>
       <c r="N11" s="22"/>
-      <c r="O11" s="22">
+      <c r="O11" s="22"/>
+      <c r="P11" s="22">
         <v>5.15</v>
       </c>
-      <c r="P11" s="22">
+      <c r="Q11" s="22">
         <v>28</v>
       </c>
-      <c r="Q11" s="13"/>
-    </row>
-    <row r="12" spans="1:18" ht="15" x14ac:dyDescent="0.25">
-      <c r="H12" s="16"/>
-    </row>
-    <row r="13" spans="1:18" ht="15" x14ac:dyDescent="0.25">
-      <c r="H13" s="16"/>
-    </row>
-    <row r="14" spans="1:18" ht="15" x14ac:dyDescent="0.25">
-      <c r="H14" s="16"/>
-    </row>
-    <row r="15" spans="1:18" ht="15" x14ac:dyDescent="0.25">
-      <c r="H15" s="16"/>
-    </row>
-    <row r="16" spans="1:18" ht="15" x14ac:dyDescent="0.25">
-      <c r="H16" s="16"/>
-    </row>
-    <row r="17" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H17" s="16"/>
-    </row>
-    <row r="18" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H18" s="16"/>
-    </row>
-    <row r="19" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H19" s="16"/>
-    </row>
-    <row r="20" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H20" s="16"/>
-    </row>
-    <row r="21" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H21" s="16"/>
-    </row>
-    <row r="22" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H22" s="16"/>
-    </row>
-    <row r="23" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H23" s="16"/>
-    </row>
-    <row r="24" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H24" s="16"/>
-    </row>
-    <row r="25" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H25" s="16"/>
-    </row>
-    <row r="26" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H26" s="16"/>
-    </row>
-    <row r="27" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H27" s="16"/>
-    </row>
-    <row r="28" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H28" s="16"/>
-    </row>
-    <row r="29" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H29" s="16"/>
-    </row>
-    <row r="30" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H30" s="16"/>
-    </row>
-    <row r="31" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H31" s="16"/>
-    </row>
-    <row r="32" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H32" s="16"/>
-    </row>
-    <row r="33" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H33" s="16"/>
-    </row>
-    <row r="34" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H34" s="16"/>
-    </row>
-    <row r="35" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H35" s="16"/>
-    </row>
-    <row r="36" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H36" s="16"/>
-    </row>
-    <row r="37" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H37" s="16"/>
-    </row>
-    <row r="38" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H38" s="16"/>
-    </row>
-    <row r="39" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H39" s="16"/>
-    </row>
-    <row r="40" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H40" s="16"/>
-    </row>
-    <row r="41" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H41" s="16"/>
-    </row>
-    <row r="42" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H42" s="16"/>
-    </row>
-    <row r="43" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H43" s="16"/>
-    </row>
-    <row r="44" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H44" s="16"/>
-    </row>
-    <row r="45" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H45" s="16"/>
+      <c r="R11" s="13"/>
+    </row>
+    <row r="12" spans="1:22" ht="15" x14ac:dyDescent="0.25">
+      <c r="I12" s="16"/>
+    </row>
+    <row r="13" spans="1:22" ht="15" x14ac:dyDescent="0.25">
+      <c r="I13" s="16"/>
+    </row>
+    <row r="14" spans="1:22" ht="15" x14ac:dyDescent="0.25">
+      <c r="I14" s="16"/>
+    </row>
+    <row r="15" spans="1:22" ht="15" x14ac:dyDescent="0.25">
+      <c r="I15" s="16"/>
+    </row>
+    <row r="16" spans="1:22" ht="15" x14ac:dyDescent="0.25">
+      <c r="I16" s="16"/>
+    </row>
+    <row r="17" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I17" s="16"/>
+    </row>
+    <row r="18" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I18" s="16"/>
+    </row>
+    <row r="19" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I19" s="16"/>
+    </row>
+    <row r="20" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I20" s="16"/>
+    </row>
+    <row r="21" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I21" s="16"/>
+    </row>
+    <row r="22" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I22" s="16"/>
+    </row>
+    <row r="23" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I23" s="16"/>
+    </row>
+    <row r="24" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I24" s="16"/>
+    </row>
+    <row r="25" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I25" s="16"/>
+    </row>
+    <row r="26" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I26" s="16"/>
+    </row>
+    <row r="27" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I27" s="16"/>
+    </row>
+    <row r="28" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I28" s="16"/>
+    </row>
+    <row r="29" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I29" s="16"/>
+    </row>
+    <row r="30" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I30" s="16"/>
+    </row>
+    <row r="31" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I31" s="16"/>
+    </row>
+    <row r="32" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I32" s="16"/>
+    </row>
+    <row r="33" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I33" s="16"/>
+    </row>
+    <row r="34" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I34" s="16"/>
+    </row>
+    <row r="35" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I35" s="16"/>
+    </row>
+    <row r="36" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I36" s="16"/>
+    </row>
+    <row r="37" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I37" s="16"/>
+    </row>
+    <row r="38" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I38" s="16"/>
+    </row>
+    <row r="39" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I39" s="16"/>
+    </row>
+    <row r="40" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I40" s="16"/>
+    </row>
+    <row r="41" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I41" s="16"/>
+    </row>
+    <row r="42" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I42" s="16"/>
+    </row>
+    <row r="43" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I43" s="16"/>
+    </row>
+    <row r="44" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I44" s="16"/>
+    </row>
+    <row r="45" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I45" s="16"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:R11">
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:S11">
     <sortCondition ref="A2:A11"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1813,7 +1891,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P45"/>
+  <dimension ref="A1:S45"/>
   <sheetFormatPr defaultColWidth="8.28515625" defaultRowHeight="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.5703125" customWidth="1"/>
@@ -1821,13 +1899,14 @@
     <col min="3" max="3" width="9.85546875" customWidth="1"/>
     <col min="4" max="4" width="6" customWidth="1"/>
     <col min="5" max="5" width="6.140625" style="1" customWidth="1"/>
-    <col min="6" max="6" width="11.42578125" style="2" customWidth="1"/>
-    <col min="7" max="7" width="10.28515625" style="2" customWidth="1"/>
-    <col min="8" max="14" width="12" customWidth="1"/>
-    <col min="15" max="15" width="32.28515625" style="2" customWidth="1"/>
+    <col min="6" max="7" width="11.42578125" style="2" customWidth="1"/>
+    <col min="8" max="8" width="13.5703125" style="2" customWidth="1"/>
+    <col min="9" max="15" width="12" customWidth="1"/>
+    <col min="16" max="16" width="32.28515625" style="2" customWidth="1"/>
+    <col min="17" max="19" width="16.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="45" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:19" ht="45" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1849,32 +1928,44 @@
       <c r="G1" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="H1" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="I1" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="7" t="s">
+      <c r="J1" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="J1" s="7" t="s">
+      <c r="K1" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="K1" s="7" t="s">
+      <c r="L1" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="L1" s="7" t="s">
+      <c r="M1" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="M1" s="7" t="s">
+      <c r="N1" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="N1" s="7" t="s">
+      <c r="O1" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="O1" s="8" t="s">
+      <c r="P1" s="8" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="2" spans="1:16" ht="15" x14ac:dyDescent="0.25">
+      <c r="Q1" s="29" t="s">
+        <v>50</v>
+      </c>
+      <c r="R1" s="29" t="s">
+        <v>51</v>
+      </c>
+      <c r="S1" s="29" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="2" spans="1:19" ht="15" x14ac:dyDescent="0.25">
       <c r="A2" s="9"/>
       <c r="B2" s="10"/>
       <c r="C2" s="9"/>
@@ -1882,16 +1973,17 @@
       <c r="E2" s="10"/>
       <c r="F2" s="12"/>
       <c r="G2" s="12"/>
-      <c r="H2" s="24"/>
-      <c r="I2" s="22"/>
+      <c r="H2" s="12"/>
+      <c r="I2" s="24"/>
       <c r="J2" s="22"/>
       <c r="K2" s="22"/>
       <c r="L2" s="22"/>
       <c r="M2" s="22"/>
       <c r="N2" s="22"/>
-      <c r="O2" s="13"/>
-    </row>
-    <row r="3" spans="1:16" ht="15" x14ac:dyDescent="0.25">
+      <c r="O2" s="22"/>
+      <c r="P2" s="13"/>
+    </row>
+    <row r="3" spans="1:19" ht="15" x14ac:dyDescent="0.25">
       <c r="A3" s="9"/>
       <c r="B3" s="10"/>
       <c r="C3" s="9"/>
@@ -1899,16 +1991,17 @@
       <c r="E3" s="10"/>
       <c r="F3" s="12"/>
       <c r="G3" s="12"/>
-      <c r="H3" s="24"/>
-      <c r="I3" s="22"/>
+      <c r="H3" s="12"/>
+      <c r="I3" s="24"/>
       <c r="J3" s="22"/>
       <c r="K3" s="22"/>
       <c r="L3" s="22"/>
       <c r="M3" s="22"/>
       <c r="N3" s="22"/>
-      <c r="O3" s="13"/>
-    </row>
-    <row r="4" spans="1:16" ht="15" x14ac:dyDescent="0.25">
+      <c r="O3" s="22"/>
+      <c r="P3" s="13"/>
+    </row>
+    <row r="4" spans="1:19" ht="15" x14ac:dyDescent="0.25">
       <c r="A4" s="9"/>
       <c r="B4" s="10"/>
       <c r="C4" s="9"/>
@@ -1916,16 +2009,17 @@
       <c r="E4" s="10"/>
       <c r="F4" s="12"/>
       <c r="G4" s="12"/>
-      <c r="H4" s="24"/>
-      <c r="I4" s="22"/>
+      <c r="H4" s="12"/>
+      <c r="I4" s="24"/>
       <c r="J4" s="22"/>
       <c r="K4" s="22"/>
       <c r="L4" s="22"/>
       <c r="M4" s="22"/>
       <c r="N4" s="22"/>
-      <c r="O4" s="13"/>
-    </row>
-    <row r="5" spans="1:16" ht="15" x14ac:dyDescent="0.25">
+      <c r="O4" s="22"/>
+      <c r="P4" s="13"/>
+    </row>
+    <row r="5" spans="1:19" ht="15" x14ac:dyDescent="0.25">
       <c r="A5" s="9"/>
       <c r="B5" s="10"/>
       <c r="C5" s="9"/>
@@ -1933,16 +2027,17 @@
       <c r="E5" s="10"/>
       <c r="F5" s="12"/>
       <c r="G5" s="12"/>
-      <c r="H5" s="24"/>
-      <c r="I5" s="22"/>
+      <c r="H5" s="12"/>
+      <c r="I5" s="24"/>
       <c r="J5" s="22"/>
       <c r="K5" s="22"/>
       <c r="L5" s="22"/>
       <c r="M5" s="22"/>
       <c r="N5" s="22"/>
-      <c r="O5" s="13"/>
-    </row>
-    <row r="6" spans="1:16" ht="15" x14ac:dyDescent="0.25">
+      <c r="O5" s="22"/>
+      <c r="P5" s="13"/>
+    </row>
+    <row r="6" spans="1:19" ht="15" x14ac:dyDescent="0.25">
       <c r="A6" s="9"/>
       <c r="B6" s="10"/>
       <c r="C6" s="9"/>
@@ -1950,16 +2045,17 @@
       <c r="E6" s="10"/>
       <c r="F6" s="12"/>
       <c r="G6" s="12"/>
-      <c r="H6" s="24"/>
-      <c r="I6" s="22"/>
+      <c r="H6" s="12"/>
+      <c r="I6" s="24"/>
       <c r="J6" s="22"/>
       <c r="K6" s="22"/>
       <c r="L6" s="22"/>
       <c r="M6" s="22"/>
       <c r="N6" s="22"/>
-      <c r="O6" s="13"/>
-    </row>
-    <row r="7" spans="1:16" ht="15" x14ac:dyDescent="0.25">
+      <c r="O6" s="22"/>
+      <c r="P6" s="13"/>
+    </row>
+    <row r="7" spans="1:19" ht="15" x14ac:dyDescent="0.25">
       <c r="A7" s="9"/>
       <c r="B7" s="10"/>
       <c r="C7" s="9"/>
@@ -1967,17 +2063,18 @@
       <c r="E7" s="10"/>
       <c r="F7" s="12"/>
       <c r="G7" s="12"/>
-      <c r="H7" s="24"/>
-      <c r="I7" s="22"/>
+      <c r="H7" s="12"/>
+      <c r="I7" s="24"/>
       <c r="J7" s="22"/>
       <c r="K7" s="22"/>
       <c r="L7" s="22"/>
       <c r="M7" s="22"/>
       <c r="N7" s="22"/>
-      <c r="O7" s="13"/>
-      <c r="P7" s="14"/>
-    </row>
-    <row r="8" spans="1:16" ht="15" x14ac:dyDescent="0.25">
+      <c r="O7" s="22"/>
+      <c r="P7" s="13"/>
+      <c r="Q7" s="14"/>
+    </row>
+    <row r="8" spans="1:19" ht="15" x14ac:dyDescent="0.25">
       <c r="A8" s="9"/>
       <c r="B8" s="10"/>
       <c r="C8" s="9"/>
@@ -1985,16 +2082,17 @@
       <c r="E8" s="10"/>
       <c r="F8" s="12"/>
       <c r="G8" s="12"/>
-      <c r="H8" s="24"/>
-      <c r="I8" s="22"/>
+      <c r="H8" s="12"/>
+      <c r="I8" s="24"/>
       <c r="J8" s="22"/>
       <c r="K8" s="22"/>
       <c r="L8" s="22"/>
       <c r="M8" s="22"/>
       <c r="N8" s="22"/>
-      <c r="O8" s="15"/>
-    </row>
-    <row r="9" spans="1:16" ht="15" x14ac:dyDescent="0.25">
+      <c r="O8" s="22"/>
+      <c r="P8" s="15"/>
+    </row>
+    <row r="9" spans="1:19" ht="15" x14ac:dyDescent="0.25">
       <c r="A9" s="9"/>
       <c r="B9" s="10"/>
       <c r="C9" s="9"/>
@@ -2002,16 +2100,17 @@
       <c r="E9" s="10"/>
       <c r="F9" s="12"/>
       <c r="G9" s="12"/>
-      <c r="H9" s="28"/>
-      <c r="I9" s="22"/>
+      <c r="H9" s="12"/>
+      <c r="I9" s="28"/>
       <c r="J9" s="22"/>
       <c r="K9" s="22"/>
       <c r="L9" s="22"/>
       <c r="M9" s="22"/>
       <c r="N9" s="22"/>
-      <c r="O9" s="27"/>
-    </row>
-    <row r="10" spans="1:16" ht="15" x14ac:dyDescent="0.25">
+      <c r="O9" s="22"/>
+      <c r="P9" s="27"/>
+    </row>
+    <row r="10" spans="1:19" ht="15" x14ac:dyDescent="0.25">
       <c r="A10" s="9"/>
       <c r="B10" s="10"/>
       <c r="C10" s="9"/>
@@ -2019,16 +2118,17 @@
       <c r="E10" s="10"/>
       <c r="F10" s="12"/>
       <c r="G10" s="12"/>
-      <c r="H10" s="24"/>
-      <c r="I10" s="22"/>
+      <c r="H10" s="12"/>
+      <c r="I10" s="24"/>
       <c r="J10" s="22"/>
       <c r="K10" s="22"/>
       <c r="L10" s="22"/>
       <c r="M10" s="22"/>
       <c r="N10" s="22"/>
-      <c r="O10" s="13"/>
-    </row>
-    <row r="11" spans="1:16" ht="15" x14ac:dyDescent="0.25">
+      <c r="O10" s="22"/>
+      <c r="P10" s="13"/>
+    </row>
+    <row r="11" spans="1:19" ht="15" x14ac:dyDescent="0.25">
       <c r="A11" s="9"/>
       <c r="B11" s="10"/>
       <c r="C11" s="9"/>
@@ -2036,120 +2136,121 @@
       <c r="E11" s="10"/>
       <c r="F11" s="12"/>
       <c r="G11" s="12"/>
-      <c r="H11" s="24"/>
-      <c r="I11" s="22"/>
+      <c r="H11" s="12"/>
+      <c r="I11" s="24"/>
       <c r="J11" s="22"/>
       <c r="K11" s="22"/>
       <c r="L11" s="22"/>
       <c r="M11" s="22"/>
       <c r="N11" s="22"/>
-      <c r="O11" s="13"/>
-    </row>
-    <row r="12" spans="1:16" ht="15" x14ac:dyDescent="0.25">
-      <c r="H12" s="16"/>
-    </row>
-    <row r="13" spans="1:16" ht="15" x14ac:dyDescent="0.25">
-      <c r="H13" s="16"/>
-    </row>
-    <row r="14" spans="1:16" ht="15" x14ac:dyDescent="0.25">
-      <c r="H14" s="16"/>
-    </row>
-    <row r="15" spans="1:16" ht="15" x14ac:dyDescent="0.25">
-      <c r="H15" s="16"/>
-    </row>
-    <row r="16" spans="1:16" ht="15" x14ac:dyDescent="0.25">
-      <c r="H16" s="16"/>
-    </row>
-    <row r="17" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H17" s="16"/>
-    </row>
-    <row r="18" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H18" s="16"/>
-    </row>
-    <row r="19" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H19" s="16"/>
-    </row>
-    <row r="20" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H20" s="16"/>
-    </row>
-    <row r="21" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H21" s="16"/>
-    </row>
-    <row r="22" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H22" s="16"/>
-    </row>
-    <row r="23" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H23" s="16"/>
-    </row>
-    <row r="24" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H24" s="16"/>
-    </row>
-    <row r="25" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H25" s="16"/>
-    </row>
-    <row r="26" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H26" s="16"/>
-    </row>
-    <row r="27" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H27" s="16"/>
-    </row>
-    <row r="28" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H28" s="16"/>
-    </row>
-    <row r="29" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H29" s="16"/>
-    </row>
-    <row r="30" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H30" s="16"/>
-    </row>
-    <row r="31" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H31" s="16"/>
-    </row>
-    <row r="32" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H32" s="16"/>
-    </row>
-    <row r="33" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H33" s="16"/>
-    </row>
-    <row r="34" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H34" s="16"/>
-    </row>
-    <row r="35" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H35" s="16"/>
-    </row>
-    <row r="36" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H36" s="16"/>
-    </row>
-    <row r="37" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H37" s="16"/>
-    </row>
-    <row r="38" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H38" s="16"/>
-    </row>
-    <row r="39" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H39" s="16"/>
-    </row>
-    <row r="40" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H40" s="16"/>
-    </row>
-    <row r="41" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H41" s="16"/>
-    </row>
-    <row r="42" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H42" s="16"/>
-    </row>
-    <row r="43" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H43" s="16"/>
-    </row>
-    <row r="44" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H44" s="16"/>
-    </row>
-    <row r="45" spans="8:8" ht="15" x14ac:dyDescent="0.25">
-      <c r="H45" s="16"/>
+      <c r="O11" s="22"/>
+      <c r="P11" s="13"/>
+    </row>
+    <row r="12" spans="1:19" ht="15" x14ac:dyDescent="0.25">
+      <c r="I12" s="16"/>
+    </row>
+    <row r="13" spans="1:19" ht="15" x14ac:dyDescent="0.25">
+      <c r="I13" s="16"/>
+    </row>
+    <row r="14" spans="1:19" ht="15" x14ac:dyDescent="0.25">
+      <c r="I14" s="16"/>
+    </row>
+    <row r="15" spans="1:19" ht="15" x14ac:dyDescent="0.25">
+      <c r="I15" s="16"/>
+    </row>
+    <row r="16" spans="1:19" ht="15" x14ac:dyDescent="0.25">
+      <c r="I16" s="16"/>
+    </row>
+    <row r="17" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I17" s="16"/>
+    </row>
+    <row r="18" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I18" s="16"/>
+    </row>
+    <row r="19" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I19" s="16"/>
+    </row>
+    <row r="20" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I20" s="16"/>
+    </row>
+    <row r="21" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I21" s="16"/>
+    </row>
+    <row r="22" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I22" s="16"/>
+    </row>
+    <row r="23" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I23" s="16"/>
+    </row>
+    <row r="24" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I24" s="16"/>
+    </row>
+    <row r="25" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I25" s="16"/>
+    </row>
+    <row r="26" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I26" s="16"/>
+    </row>
+    <row r="27" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I27" s="16"/>
+    </row>
+    <row r="28" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I28" s="16"/>
+    </row>
+    <row r="29" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I29" s="16"/>
+    </row>
+    <row r="30" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I30" s="16"/>
+    </row>
+    <row r="31" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I31" s="16"/>
+    </row>
+    <row r="32" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I32" s="16"/>
+    </row>
+    <row r="33" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I33" s="16"/>
+    </row>
+    <row r="34" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I34" s="16"/>
+    </row>
+    <row r="35" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I35" s="16"/>
+    </row>
+    <row r="36" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I36" s="16"/>
+    </row>
+    <row r="37" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I37" s="16"/>
+    </row>
+    <row r="38" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I38" s="16"/>
+    </row>
+    <row r="39" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I39" s="16"/>
+    </row>
+    <row r="40" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I40" s="16"/>
+    </row>
+    <row r="41" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I41" s="16"/>
+    </row>
+    <row r="42" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I42" s="16"/>
+    </row>
+    <row r="43" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I43" s="16"/>
+    </row>
+    <row r="44" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I44" s="16"/>
+    </row>
+    <row r="45" spans="9:9" ht="15" x14ac:dyDescent="0.25">
+      <c r="I45" s="16"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup fitToHeight="0" orientation="landscape" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup fitToHeight="0" orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Refactored to reduce use of _col_letter() and minor formatting changes
</commit_message>
<xml_diff>
--- a/Testing/basic_sequence/workbook.xlsx
+++ b/Testing/basic_sequence/workbook.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Pavan Rauch\git\Truancy-Local\Testing\basic_sequence\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{098948B8-56D6-45A8-8784-CC0EE9BD252B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8957103D-4B30-49C9-9B0D-E7E468AB15BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Urbana Elementary (Before)" sheetId="4" r:id="rId1"/>
@@ -1487,6 +1487,9 @@
       <c r="R5" s="13" t="s">
         <v>33</v>
       </c>
+      <c r="S5" s="30">
+        <v>45672</v>
+      </c>
     </row>
     <row r="6" spans="1:22" ht="15" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
@@ -1586,6 +1589,12 @@
       </c>
       <c r="R7" s="13" t="s">
         <v>35</v>
+      </c>
+      <c r="S7" s="30">
+        <v>45664</v>
+      </c>
+      <c r="T7" s="30">
+        <v>45680</v>
       </c>
       <c r="V7" s="14" t="s">
         <v>32</v>

</xml_diff>